<commit_message>
before storing manual mapping an stored all filetype securities
</commit_message>
<xml_diff>
--- a/evaluation_results.xlsx
+++ b/evaluation_results.xlsx
@@ -584,19 +584,19 @@
         <v>1</v>
       </c>
       <c r="P2" t="n">
-        <v>0.9293</v>
+        <v>1</v>
       </c>
       <c r="Q2" t="n">
-        <v>263.8432</v>
+        <v>1</v>
       </c>
       <c r="R2" t="inlineStr">
         <is>
-          <t>360DG | Watchtower Buyer | Marketplace Events | APRA | APHIX</t>
+          <t>360DG</t>
         </is>
       </c>
       <c r="S2" t="inlineStr">
         <is>
-          <t>360DG (Term Loan) | 360DG (DDTL B) | 360DG (DDTL A) | 360DG (Revolver) | 360DG (Common Equity)</t>
+          <t>360DG (Term Loan)</t>
         </is>
       </c>
       <c r="T2" t="b">
@@ -671,16 +671,16 @@
         <v>1</v>
       </c>
       <c r="Q3" t="n">
-        <v>286.0734</v>
+        <v>1</v>
       </c>
       <c r="R3" t="inlineStr">
         <is>
-          <t>48Forty | Smartronix / Trident | Altamira | Douglas | Engine &amp; Transmission Exchange</t>
+          <t>48Forty</t>
         </is>
       </c>
       <c r="S3" t="inlineStr">
         <is>
-          <t>48Forty (Common Equity) | 48Forty (Term Loan) | Smartronix / Trident (TL) | 48Forty (DDTL) | Altamira (Common Equity)</t>
+          <t>48Forty (Common Equity)</t>
         </is>
       </c>
       <c r="T3" t="b">
@@ -755,16 +755,16 @@
         <v>1</v>
       </c>
       <c r="Q4" t="n">
-        <v>463.4119</v>
+        <v>1</v>
       </c>
       <c r="R4" t="inlineStr">
         <is>
-          <t>Ad.net | Arcfield | C5MI | Duggal Visual Solutions | GCOM</t>
+          <t>Ad.net</t>
         </is>
       </c>
       <c r="S4" t="inlineStr">
         <is>
-          <t>Ad.net (Term Loan) | Ad.net (Revolver) | Ad.net (Common Equity) | Ad.net (Preferred Equity) | Arcfield (Term Loan)</t>
+          <t>Ad.net (Term Loan)</t>
         </is>
       </c>
       <c r="T4" t="b">
@@ -839,16 +839,16 @@
         <v>1</v>
       </c>
       <c r="Q5" t="n">
-        <v>425.9401</v>
+        <v>1</v>
       </c>
       <c r="R5" t="inlineStr">
         <is>
-          <t>Aechelon | Intellectual Technology | Sabel Systems</t>
+          <t>Aechelon</t>
         </is>
       </c>
       <c r="S5" t="inlineStr">
         <is>
-          <t>Aechelon (Term Loan) | Aechelon (Revolver) | Aechelon (Common Equity) | Intellectual Technology, Inc. (TL) | Sabel Systems (Term Loan)</t>
+          <t>Aechelon (Term Loan)</t>
         </is>
       </c>
       <c r="T5" t="b">
@@ -920,19 +920,19 @@
         <v>1</v>
       </c>
       <c r="P6" t="n">
-        <v>0.8579</v>
+        <v>1</v>
       </c>
       <c r="Q6" t="n">
-        <v>314.2243</v>
+        <v>1</v>
       </c>
       <c r="R6" t="inlineStr">
         <is>
-          <t>AFC Acquisitions | Watchtower Holdings</t>
+          <t>AFC Acquisitions</t>
         </is>
       </c>
       <c r="S6" t="inlineStr">
         <is>
-          <t>AFC Industries (DDTL) | AFC Industries (Common Equity) | AFC Industries (TL) | Watchtower Holding (Common Equity)</t>
+          <t>AFC Industries (DDTL)</t>
         </is>
       </c>
       <c r="T6" t="b">
@@ -1004,19 +1004,19 @@
         <v>1</v>
       </c>
       <c r="P7" t="n">
-        <v>0.8579</v>
+        <v>1</v>
       </c>
       <c r="Q7" t="n">
-        <v>230.7481</v>
+        <v>1</v>
       </c>
       <c r="R7" t="inlineStr">
         <is>
-          <t>AFC Acquisitions | Watchtower Holdings</t>
+          <t>AFC Acquisitions</t>
         </is>
       </c>
       <c r="S7" t="inlineStr">
         <is>
-          <t>AFC Industries (TL) | AFC Industries (DDTL) | AFC Industries (Common Equity) | Watchtower Holding (Common Equity)</t>
+          <t>AFC Industries (TL)</t>
         </is>
       </c>
       <c r="T7" t="b">
@@ -1091,16 +1091,16 @@
         <v>1</v>
       </c>
       <c r="Q8" t="n">
-        <v>621.1671</v>
+        <v>1</v>
       </c>
       <c r="R8" t="inlineStr">
         <is>
-          <t>BBB Industries | STG Logistics | Adweek | Aspect Software | Health-E Commerce</t>
+          <t>BBB Industries</t>
         </is>
       </c>
       <c r="S8" t="inlineStr">
         <is>
-          <t>BBB Industries (First Lien Term Loan) | BBB Industries (Second Lien Term Loan) | STG (TL) | Adweek (Term Loan) | Adweek (DDTL)</t>
+          <t>BBB Industries (First Lien Term Loan)</t>
         </is>
       </c>
       <c r="T8" t="b">
@@ -1175,7 +1175,7 @@
         <v>0.9023</v>
       </c>
       <c r="Q9" t="n">
-        <v>423.274</v>
+        <v>605.7479</v>
       </c>
       <c r="R9" t="inlineStr">
         <is>
@@ -1259,16 +1259,16 @@
         <v>1</v>
       </c>
       <c r="Q10" t="n">
-        <v>344.7419</v>
+        <v>1</v>
       </c>
       <c r="R10" t="inlineStr">
         <is>
-          <t>Bluebird | The Creative Group | The Original Cakerie | Simplicity Group | None</t>
+          <t>Bluebird</t>
         </is>
       </c>
       <c r="S10" t="inlineStr">
         <is>
-          <t>Bluebird (Term Loan) | Bluebird (Revolver) | Simplicity Group (TL) | The Creative Group (Term Loan) | Simplicity Group (DDTL)</t>
+          <t>Bluebird (Term Loan)</t>
         </is>
       </c>
       <c r="T10" t="b">
@@ -1340,19 +1340,19 @@
         <v>1</v>
       </c>
       <c r="P11" t="n">
-        <v>0.9736</v>
+        <v>1</v>
       </c>
       <c r="Q11" t="n">
-        <v>587.9376</v>
+        <v>1</v>
       </c>
       <c r="R11" t="inlineStr">
         <is>
-          <t>BlueHalo | API Technologies | Altamira | Nuvei | Lynx Technologies</t>
+          <t>BlueHalo</t>
         </is>
       </c>
       <c r="S11" t="inlineStr">
         <is>
-          <t>BlueHalo (Term Loan) | API Technologies (TL) | API Technologies (Revolver) | Altamira (Common Equity) | Altamira (TL)</t>
+          <t>BlueHalo (Term Loan)</t>
         </is>
       </c>
       <c r="T11" t="b">
@@ -1392,51 +1392,55 @@
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>Global</t>
+          <t>BlueHalo</t>
         </is>
       </c>
       <c r="H12" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I12" t="b">
         <v>1</v>
       </c>
       <c r="J12" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K12" t="inlineStr">
         <is>
           <t>BlueHalo (Term Loan)</t>
         </is>
       </c>
-      <c r="L12" t="inlineStr"/>
+      <c r="L12" t="inlineStr">
+        <is>
+          <t>BlueHalo (Term Loan)</t>
+        </is>
+      </c>
       <c r="M12" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="N12" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O12" t="n">
-        <v>8</v>
+        <v>1</v>
       </c>
       <c r="P12" t="n">
-        <v>0.8575</v>
+        <v>1</v>
       </c>
       <c r="Q12" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="R12" t="inlineStr">
         <is>
-          <t>Global | BlueHalo | Insight Global | Schlesinger | UniTek</t>
+          <t>BlueHalo</t>
         </is>
       </c>
       <c r="S12" t="inlineStr">
         <is>
-          <t>Schlesinger (Term Loan) | Schlesinger (Equity) | Global (Term Loan) | Insight Global (TL) | Insight Global (Rev)</t>
+          <t>BlueHalo (Term Loan)</t>
         </is>
       </c>
       <c r="T12" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="13">
@@ -1507,16 +1511,16 @@
         <v>1</v>
       </c>
       <c r="Q13" t="n">
-        <v>465.409</v>
+        <v>1</v>
       </c>
       <c r="R13" t="inlineStr">
         <is>
-          <t>By Light | Integrated Data Services | Any Hour Services | Applied Technical Services | IDC Infusion Services</t>
+          <t>By Light</t>
         </is>
       </c>
       <c r="S13" t="inlineStr">
         <is>
-          <t>By Light (Revolver) | By Light (Term Loan) | By Light (DDTL) | By Light (Equity) | By Light (HoldCo Note)</t>
+          <t>By Light (Revolver)</t>
         </is>
       </c>
       <c r="T13" t="b">
@@ -1591,7 +1595,7 @@
         <v>0.9533</v>
       </c>
       <c r="Q14" t="n">
-        <v>247.061</v>
+        <v>345.8854</v>
       </c>
       <c r="R14" t="inlineStr">
         <is>
@@ -1600,7 +1604,7 @@
       </c>
       <c r="S14" t="inlineStr">
         <is>
-          <t>Centauri Health (TL) | Centauri Health (Revolver) | Centauri Health (DDTL) | Watchtower Buyer (Revolver) | Carisk Partners (Revolver)</t>
+          <t>Centauri Health (TL) | Centauri Health (Revolver) | Watchtower Buyer (Revolver) | Centauri Health (DDTL) | Carisk Partners (Revolver)</t>
         </is>
       </c>
       <c r="T14" t="b">
@@ -1675,16 +1679,16 @@
         <v>1</v>
       </c>
       <c r="Q15" t="n">
-        <v>392.2633</v>
+        <v>1</v>
       </c>
       <c r="R15" t="inlineStr">
         <is>
-          <t>Dr. Squatch | Dr. Scholl's</t>
+          <t>Dr. Squatch</t>
         </is>
       </c>
       <c r="S15" t="inlineStr">
         <is>
-          <t>Dr. Squatch (Term Loan) | Dr. Squatch (Revolver) | Dr. Squatch (DDTL) | Dr. Scholl's (Term Loan) | Dr. Scholl's (Revolver)</t>
+          <t>Dr. Squatch (Term Loan)</t>
         </is>
       </c>
       <c r="T15" t="b">
@@ -1756,19 +1760,19 @@
         <v>1</v>
       </c>
       <c r="P16" t="n">
-        <v>0.9911</v>
+        <v>1</v>
       </c>
       <c r="Q16" t="n">
-        <v>438.3659</v>
+        <v>1</v>
       </c>
       <c r="R16" t="inlineStr">
         <is>
-          <t>Guild Garage Group | PCS Retirement | Total Pool Care Network</t>
+          <t>Guild Garage Group</t>
         </is>
       </c>
       <c r="S16" t="inlineStr">
         <is>
-          <t>Guild Garage Group (DDTL) | Guild Garage Group (Term Loan) | TPCN (DDTL) | PCS Retirement (DDTL) | TPCN (Term Loan)</t>
+          <t>Guild Garage Group (DDTL)</t>
         </is>
       </c>
       <c r="T16" t="b">
@@ -1843,16 +1847,16 @@
         <v>1</v>
       </c>
       <c r="Q17" t="n">
-        <v>516.9478</v>
+        <v>1</v>
       </c>
       <c r="R17" t="inlineStr">
         <is>
-          <t>Infinity Home Services | United Land Services | Any Hour Services | Applied Technical Services | IDC Infusion Services</t>
+          <t>Infinity Home Services</t>
         </is>
       </c>
       <c r="S17" t="inlineStr">
         <is>
-          <t>Infinity Home Services (DDTL) | Infinity Home Services (DDTL) CAD | Infinity Home Services (Term Loan) | United Land Services (HoldCo Notes DDTL) | Any Hour Services (DDTL)</t>
+          <t>Infinity Home Services (DDTL)</t>
         </is>
       </c>
       <c r="T17" t="b">
@@ -1924,19 +1928,19 @@
         <v>1</v>
       </c>
       <c r="P18" t="n">
-        <v>0.9896</v>
+        <v>1</v>
       </c>
       <c r="Q18" t="n">
-        <v>350.5145</v>
+        <v>1</v>
       </c>
       <c r="R18" t="inlineStr">
         <is>
-          <t>Lilly Lashes | APT Healthcare | Zips</t>
+          <t>Lilly Lashes</t>
         </is>
       </c>
       <c r="S18" t="inlineStr">
         <is>
-          <t>Lilly Lashes (TL) | APT Healthcare (Term Loan) | APT Healthcare (Incr. DDTL) | Zips (New OpCo Term Loan) | APT Healthcare (Common Equity)</t>
+          <t>Lilly Lashes (TL)</t>
         </is>
       </c>
       <c r="T18" t="b">
@@ -2011,16 +2015,16 @@
         <v>1</v>
       </c>
       <c r="Q19" t="n">
-        <v>446.1023</v>
+        <v>1</v>
       </c>
       <c r="R19" t="inlineStr">
         <is>
-          <t>Lynx Technologies | PAR Excellence | STG Logistics | Adweek | Aspect Software</t>
+          <t>Lynx Technologies</t>
         </is>
       </c>
       <c r="S19" t="inlineStr">
         <is>
-          <t>Lynx Technologies (TL) | STG (TL) | Adweek (Term Loan) | Adweek (DDTL) | Aspect Software (Equity)</t>
+          <t>Lynx Technologies (TL)</t>
         </is>
       </c>
       <c r="T19" t="b">
@@ -2092,10 +2096,10 @@
         <v>1</v>
       </c>
       <c r="P20" t="n">
-        <v>0.8696</v>
+        <v>1</v>
       </c>
       <c r="Q20" t="n">
-        <v>360.7486</v>
+        <v>1</v>
       </c>
       <c r="R20" t="inlineStr">
         <is>
@@ -2104,7 +2108,7 @@
       </c>
       <c r="S20" t="inlineStr">
         <is>
-          <t>MeritDirect (Term Loan) | MeritDirect (Common Equity) | MeritDirect (Preferred Equity) | MeritDirect (Revolver)</t>
+          <t>MeritDirect (Term Loan)</t>
         </is>
       </c>
       <c r="T20" t="b">
@@ -2179,7 +2183,7 @@
         <v>1</v>
       </c>
       <c r="Q21" t="n">
-        <v>454.5237</v>
+        <v>1</v>
       </c>
       <c r="R21" t="inlineStr">
         <is>
@@ -2188,7 +2192,7 @@
       </c>
       <c r="S21" t="inlineStr">
         <is>
-          <t>MeritDirect (Term Loan) | MeritDirect (Common Equity) | MeritDirect (Preferred Equity) | MeritDirect (Revolver)</t>
+          <t>MeritDirect (Term Loan)</t>
         </is>
       </c>
       <c r="T21" t="b">
@@ -2245,19 +2249,25 @@
           <t>OSG (Common Equity)</t>
         </is>
       </c>
-      <c r="L22" t="inlineStr"/>
+      <c r="L22" t="inlineStr">
+        <is>
+          <t>U.S. Well (Class A)</t>
+        </is>
+      </c>
       <c r="M22" t="b">
         <v>0</v>
       </c>
       <c r="N22" t="b">
-        <v>0</v>
-      </c>
-      <c r="O22" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="O22" t="n">
+        <v>5</v>
+      </c>
       <c r="P22" t="n">
-        <v>0.8529</v>
+        <v>0.8549</v>
       </c>
       <c r="Q22" t="n">
-        <v>0</v>
+        <v>85.36020000000001</v>
       </c>
       <c r="R22" t="inlineStr">
         <is>
@@ -2266,11 +2276,11 @@
       </c>
       <c r="S22" t="inlineStr">
         <is>
-          <t>A1 Garage (DDTL) | AKW Holdings (Term Loan) | AKW Holdings (Common) | Learning Care Group (Common) | CEA (Common)</t>
+          <t>U.S. Well (Class A) | Imagine Topco. L.P. (Preferred Equity - Series A) | U.S. Well (Class B) | Superior (Preferred A) | OSG (Common Equity)</t>
         </is>
       </c>
       <c r="T22" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="23">
@@ -2323,9 +2333,13 @@
           <t>Pragmatic Institute (Common)</t>
         </is>
       </c>
-      <c r="L23" t="inlineStr"/>
+      <c r="L23" t="inlineStr">
+        <is>
+          <t>Pragmatic Institute (Common)</t>
+        </is>
+      </c>
       <c r="M23" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="N23" t="b">
         <v>1</v>
@@ -2337,7 +2351,7 @@
         <v>1</v>
       </c>
       <c r="Q23" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="R23" t="inlineStr">
         <is>
@@ -2346,11 +2360,11 @@
       </c>
       <c r="S23" t="inlineStr">
         <is>
-          <t>Pragmatic Institute (Common) | Pragmatic Institute (TL) | Pragmatic Institute (Revolver) | Pragmatic Institute (DDTL)</t>
+          <t>Pragmatic Institute (Common)</t>
         </is>
       </c>
       <c r="T23" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="24">
@@ -2421,7 +2435,7 @@
         <v>1</v>
       </c>
       <c r="Q24" t="n">
-        <v>423.655</v>
+        <v>1</v>
       </c>
       <c r="R24" t="inlineStr">
         <is>
@@ -2430,7 +2444,7 @@
       </c>
       <c r="S24" t="inlineStr">
         <is>
-          <t>C&amp;K Paving Contractors (Term Loan) | C&amp;K Paving Contractors (DDTL) | C&amp;K Paving Contractors (Common Equity)</t>
+          <t>C&amp;K Paving Contractors (Term Loan)</t>
         </is>
       </c>
       <c r="T24" t="b">
@@ -2496,19 +2510,19 @@
       </c>
       <c r="O25" t="inlineStr"/>
       <c r="P25" t="n">
-        <v>0.9533</v>
+        <v>1</v>
       </c>
       <c r="Q25" t="n">
-        <v>293.4885</v>
+        <v>1</v>
       </c>
       <c r="R25" t="inlineStr">
         <is>
-          <t>Centauri Health | Watchtower Buyer | APHIX | Carisk Partners | Connatix</t>
+          <t>Centauri Health</t>
         </is>
       </c>
       <c r="S25" t="inlineStr">
         <is>
-          <t>Centauri Health (TL) | Centauri Health (DDTL) | Centauri Health (Revolver) | Watchtower Buyer (TL) | Watchtower Buyer (DDTL)</t>
+          <t>Centauri Health (TL)</t>
         </is>
       </c>
       <c r="T25" t="b">
@@ -2580,19 +2594,19 @@
         <v>1</v>
       </c>
       <c r="P26" t="n">
-        <v>0.9834000000000001</v>
+        <v>1</v>
       </c>
       <c r="Q26" t="n">
-        <v>381.1502</v>
+        <v>1</v>
       </c>
       <c r="R26" t="inlineStr">
         <is>
-          <t>Commercial Fire Protection | AKW Holdings</t>
+          <t>Commercial Fire Protection</t>
         </is>
       </c>
       <c r="S26" t="inlineStr">
         <is>
-          <t>Commercial Fire Protection (Term Loan) | Commercial Fire Protection (DDTL) | Commercial Fire Protection (Revolver) | Commercial Fire Protection (Common Equity) | AKW Holdings (Term Loan)</t>
+          <t>Commercial Fire Protection (Term Loan)</t>
         </is>
       </c>
       <c r="T26" t="b">
@@ -2664,19 +2678,19 @@
         <v>1</v>
       </c>
       <c r="P27" t="n">
-        <v>0.8377</v>
+        <v>1</v>
       </c>
       <c r="Q27" t="n">
-        <v>349.8867</v>
+        <v>1</v>
       </c>
       <c r="R27" t="inlineStr">
         <is>
-          <t>Dr. Scholl's | Apex Service Partners | API Technologies | Wheel Pros | Paris Presents</t>
+          <t>Dr. Scholl's</t>
         </is>
       </c>
       <c r="S27" t="inlineStr">
         <is>
-          <t>Dr. Scholl's (Term Loan) | API Technologies (TL) | API Technologies (Revolver) | Apex (Term Loan) | Apex (Incremental Term Loan)</t>
+          <t>Dr. Scholl's (Term Loan)</t>
         </is>
       </c>
       <c r="T27" t="b">
@@ -2731,7 +2745,11 @@
           <t>Fairbanks Morse Defense (Term Loan)</t>
         </is>
       </c>
-      <c r="L28" t="inlineStr"/>
+      <c r="L28" t="inlineStr">
+        <is>
+          <t>AKW Holdings (Term Loan)</t>
+        </is>
+      </c>
       <c r="M28" t="b">
         <v>0</v>
       </c>
@@ -2740,10 +2758,10 @@
       </c>
       <c r="O28" t="inlineStr"/>
       <c r="P28" t="n">
-        <v>0.6244</v>
+        <v>0.6002999999999999</v>
       </c>
       <c r="Q28" t="n">
-        <v>0</v>
+        <v>36.3303</v>
       </c>
       <c r="R28" t="inlineStr">
         <is>
@@ -2756,7 +2774,7 @@
         </is>
       </c>
       <c r="T28" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="29">
@@ -2827,16 +2845,16 @@
         <v>1</v>
       </c>
       <c r="Q29" t="n">
-        <v>466.0747</v>
+        <v>1</v>
       </c>
       <c r="R29" t="inlineStr">
         <is>
-          <t>MCR | Research Now/SSI | PhaseWell Research | Pinnacle Clinical Research | CHA Consulting</t>
+          <t>MCR</t>
         </is>
       </c>
       <c r="S29" t="inlineStr">
         <is>
-          <t>MCR (Term Loan) | MCR (Revolver) | CHA Consulting (TL) | CHA Consulting (DDTL) | Research Now / SSI (Common Equity)</t>
+          <t>MCR (Term Loan)</t>
         </is>
       </c>
       <c r="T29" t="b">
@@ -2907,7 +2925,7 @@
         <v>1</v>
       </c>
       <c r="Q30" t="n">
-        <v>324.8272</v>
+        <v>432.755</v>
       </c>
       <c r="R30" t="inlineStr">
         <is>
@@ -2991,7 +3009,7 @@
         <v>1</v>
       </c>
       <c r="Q31" t="n">
-        <v>324.8272</v>
+        <v>1</v>
       </c>
       <c r="R31" t="inlineStr">
         <is>
@@ -3069,13 +3087,13 @@
         <v>0</v>
       </c>
       <c r="O32" t="n">
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="P32" t="n">
         <v>0.7469</v>
       </c>
       <c r="Q32" t="n">
-        <v>270.9943</v>
+        <v>391.6117</v>
       </c>
       <c r="R32" t="inlineStr">
         <is>
@@ -3084,7 +3102,7 @@
       </c>
       <c r="S32" t="inlineStr">
         <is>
-          <t>APT Healthcare (Incr. DDTL) | Zips (DDTL) | APT Healthcare (Term Loan) | APT Healthcare (Common Equity) | APT Healthcare (Revolver)</t>
+          <t>APT Healthcare (Incr. DDTL) | Zips (DDTL) | APT Healthcare (Term Loan) | Lilly Lashes (TL) | APT Healthcare (Common Equity)</t>
         </is>
       </c>
       <c r="T32" t="b">
@@ -3152,10 +3170,10 @@
       </c>
       <c r="O33" t="inlineStr"/>
       <c r="P33" t="n">
-        <v>0.8356</v>
+        <v>0.8365</v>
       </c>
       <c r="Q33" t="n">
-        <v>265.6984</v>
+        <v>394.7907</v>
       </c>
       <c r="R33" t="inlineStr">
         <is>
@@ -3236,10 +3254,10 @@
         <v>1</v>
       </c>
       <c r="P34" t="n">
-        <v>1</v>
+        <v>0.9995000000000001</v>
       </c>
       <c r="Q34" t="n">
-        <v>429.7589</v>
+        <v>618.7388999999999</v>
       </c>
       <c r="R34" t="inlineStr">
         <is>
@@ -3323,7 +3341,7 @@
         <v>0.9834000000000001</v>
       </c>
       <c r="Q35" t="n">
-        <v>384.8888</v>
+        <v>537.6147</v>
       </c>
       <c r="R35" t="inlineStr">
         <is>
@@ -3332,7 +3350,7 @@
       </c>
       <c r="S35" t="inlineStr">
         <is>
-          <t>4Wall Entertainment (Term Loan) | 4Wall Entertainment (DDTL) | AKW Holdings (Term Loan) | AKW Holdings (Common) | 4Wall Entertainment (Revolver)</t>
+          <t>4Wall Entertainment (Term Loan) | 4Wall Entertainment (DDTL) | 4Wall Entertainment (Revolver) | AKW Holdings (Term Loan) | AKW Holdings (Common)</t>
         </is>
       </c>
       <c r="T35" t="b">
@@ -3407,7 +3425,7 @@
         <v>1</v>
       </c>
       <c r="Q36" t="n">
-        <v>505.2237</v>
+        <v>706.376</v>
       </c>
       <c r="R36" t="inlineStr">
         <is>
@@ -3491,7 +3509,7 @@
         <v>1</v>
       </c>
       <c r="Q37" t="n">
-        <v>445.7695</v>
+        <v>658.7212</v>
       </c>
       <c r="R37" t="inlineStr">
         <is>
@@ -3559,23 +3577,23 @@
       </c>
       <c r="L38" t="inlineStr">
         <is>
-          <t>BlueHalo (Term Loan)</t>
+          <t>Global (Term Loan)</t>
         </is>
       </c>
       <c r="M38" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="N38" t="b">
         <v>1</v>
       </c>
       <c r="O38" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="P38" t="n">
-        <v>0.8575</v>
+        <v>0.8559</v>
       </c>
       <c r="Q38" t="n">
-        <v>268.6741</v>
+        <v>374.5238</v>
       </c>
       <c r="R38" t="inlineStr">
         <is>
@@ -3584,7 +3602,7 @@
       </c>
       <c r="S38" t="inlineStr">
         <is>
-          <t>BlueHalo (Term Loan) | Global (Term Loan) | Insight Global (TL) | Schlesinger (Term Loan) | Schlesinger (DDTL)</t>
+          <t>Global (Term Loan) | BlueHalo (Term Loan) | Insight Global (TL) | Schlesinger (Term Loan) | Schlesinger (DDTL)</t>
         </is>
       </c>
       <c r="T38" t="b">
@@ -3659,7 +3677,7 @@
         <v>1</v>
       </c>
       <c r="Q39" t="n">
-        <v>408.6695</v>
+        <v>571.072</v>
       </c>
       <c r="R39" t="inlineStr">
         <is>
@@ -3743,7 +3761,7 @@
         <v>0.9758</v>
       </c>
       <c r="Q40" t="n">
-        <v>328.7208</v>
+        <v>458.7628</v>
       </c>
       <c r="R40" t="inlineStr">
         <is>
@@ -3827,7 +3845,7 @@
         <v>1</v>
       </c>
       <c r="Q41" t="n">
-        <v>437.8485</v>
+        <v>649.8196</v>
       </c>
       <c r="R41" t="inlineStr">
         <is>
@@ -3911,7 +3929,7 @@
         <v>1</v>
       </c>
       <c r="Q42" t="n">
-        <v>382.8196</v>
+        <v>538.772</v>
       </c>
       <c r="R42" t="inlineStr">
         <is>
@@ -3991,7 +4009,7 @@
         <v>0.7544</v>
       </c>
       <c r="Q43" t="n">
-        <v>270.3769</v>
+        <v>391.6918</v>
       </c>
       <c r="R43" t="inlineStr">
         <is>
@@ -4000,7 +4018,7 @@
       </c>
       <c r="S43" t="inlineStr">
         <is>
-          <t>US Fertility (DDTL) | TVC (DDTL) | TVC (TL) | US Fertility (Term Loan) | TVC (Equity)</t>
+          <t>US Fertility (DDTL) | TVC (DDTL) | TVC (TL) | US Fertility (Term Loan) | TVC (Revolver)</t>
         </is>
       </c>
       <c r="T43" t="b">
@@ -4071,7 +4089,7 @@
         <v>0.7544</v>
       </c>
       <c r="Q44" t="n">
-        <v>206.7704</v>
+        <v>292.8177</v>
       </c>
       <c r="R44" t="inlineStr">
         <is>
@@ -4080,7 +4098,7 @@
       </c>
       <c r="S44" t="inlineStr">
         <is>
-          <t>TVC (TL) | US Fertility (Term Loan) | US Fertility (DDTL) | TVC (DDTL) | TVC (Equity)</t>
+          <t>TVC (TL) | US Fertility (Term Loan) | US Fertility (DDTL) | TVC (DDTL) | TVC (Revolver)</t>
         </is>
       </c>
       <c r="T44" t="b">
@@ -4155,7 +4173,7 @@
         <v>0.999</v>
       </c>
       <c r="Q45" t="n">
-        <v>419.8098</v>
+        <v>590.5582000000001</v>
       </c>
       <c r="R45" t="inlineStr">
         <is>
@@ -4164,7 +4182,7 @@
       </c>
       <c r="S45" t="inlineStr">
         <is>
-          <t>Aeronix (DDTL) | Aeronix (Common Equity) | AKW Holdings (Term Loan) | Aeronix (TL) | Aeronix (Revolver)</t>
+          <t>Aeronix (DDTL) | Aeronix (Common Equity) | AKW Holdings (Term Loan) | Aeronix (TL) | AKW Holdings (Common)</t>
         </is>
       </c>
       <c r="T45" t="b">
@@ -4239,7 +4257,7 @@
         <v>0.8377</v>
       </c>
       <c r="Q46" t="n">
-        <v>349.8867</v>
+        <v>488.6119</v>
       </c>
       <c r="R46" t="inlineStr">
         <is>
@@ -4323,7 +4341,7 @@
         <v>0.8461</v>
       </c>
       <c r="Q47" t="n">
-        <v>417.5949</v>
+        <v>583.1864</v>
       </c>
       <c r="R47" t="inlineStr">
         <is>
@@ -4400,10 +4418,10 @@
       </c>
       <c r="O48" t="inlineStr"/>
       <c r="P48" t="n">
-        <v>0.549</v>
+        <v>0.5482</v>
       </c>
       <c r="Q48" t="n">
-        <v>157.2802</v>
+        <v>233.9925</v>
       </c>
       <c r="R48" t="inlineStr">
         <is>
@@ -4481,13 +4499,13 @@
         <v>1</v>
       </c>
       <c r="O49" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="P49" t="n">
-        <v>0.7583</v>
+        <v>0.76</v>
       </c>
       <c r="Q49" t="n">
-        <v>582.932</v>
+        <v>887.1277</v>
       </c>
       <c r="R49" t="inlineStr">
         <is>
@@ -4496,7 +4514,7 @@
       </c>
       <c r="S49" t="inlineStr">
         <is>
-          <t>STG (First Out New Money Term Loans) | STG (TL) | BlackHawk Industrial (Incremental TL) | BlackHawk Industrial (TL) | BlackHawk Industrial (Revolver)</t>
+          <t>STG (First Out New Money Term Loans) | STG (Second Out Term Loans) | STG (TL) | Plimpton &amp; Hills (TL) | Plimpton &amp; Hills (DDTL)</t>
         </is>
       </c>
       <c r="T49" t="b">
@@ -4571,7 +4589,7 @@
         <v>1</v>
       </c>
       <c r="Q50" t="n">
-        <v>461.5108</v>
+        <v>667.8467000000001</v>
       </c>
       <c r="R50" t="inlineStr">
         <is>
@@ -4655,7 +4673,7 @@
         <v>0.9834000000000001</v>
       </c>
       <c r="Q51" t="n">
-        <v>384.8888</v>
+        <v>537.6147</v>
       </c>
       <c r="R51" t="inlineStr">
         <is>
@@ -4664,7 +4682,7 @@
       </c>
       <c r="S51" t="inlineStr">
         <is>
-          <t>4Wall Entertainment (Term Loan) | 4Wall Entertainment (DDTL) | AKW Holdings (Term Loan) | AKW Holdings (Common) | 4Wall Entertainment (Revolver)</t>
+          <t>4Wall Entertainment (Term Loan) | 4Wall Entertainment (DDTL) | 4Wall Entertainment (Revolver) | AKW Holdings (Term Loan) | AKW Holdings (Common)</t>
         </is>
       </c>
       <c r="T51" t="b">
@@ -4736,14 +4754,14 @@
         <v>1</v>
       </c>
       <c r="P52" t="n">
-        <v>1.2</v>
+        <v>1</v>
       </c>
       <c r="Q52" t="n">
-        <v>459.0776</v>
+        <v>688.3133</v>
       </c>
       <c r="R52" t="inlineStr">
         <is>
-          <t>A1 Garage | Guild Garage Group | A2 Garge | None | Omnia</t>
+          <t>A1 Garage | A2 Garge | None | Guild Garage Group | Omnia</t>
         </is>
       </c>
       <c r="S52" t="inlineStr">
@@ -4823,7 +4841,7 @@
         <v>1</v>
       </c>
       <c r="Q53" t="n">
-        <v>471.6733</v>
+        <v>709.112</v>
       </c>
       <c r="R53" t="inlineStr">
         <is>
@@ -4907,7 +4925,7 @@
         <v>1</v>
       </c>
       <c r="Q54" t="n">
-        <v>567.4974999999999</v>
+        <v>820.9715</v>
       </c>
       <c r="R54" t="inlineStr">
         <is>
@@ -4916,7 +4934,7 @@
       </c>
       <c r="S54" t="inlineStr">
         <is>
-          <t>Beta+ (TL) | Altamira (TL) | Nuvei (Term Loan) | API Technologies (TL) | Lynx Technologies (TL)</t>
+          <t>Beta+ (TL) | API Technologies (TL) | Lynx Technologies (TL) | Altamira (TL) | Nuvei (Term Loan)</t>
         </is>
       </c>
       <c r="T54" t="b">
@@ -4991,7 +5009,7 @@
         <v>0.9499</v>
       </c>
       <c r="Q55" t="n">
-        <v>294.7243</v>
+        <v>411.894</v>
       </c>
       <c r="R55" t="inlineStr">
         <is>
@@ -5000,7 +5018,7 @@
       </c>
       <c r="S55" t="inlineStr">
         <is>
-          <t>Sparq (TL) | AKW Holdings (Term Loan) | AKW Holdings (Common) | Sparq (Common Equity) | Sparq (DDTL)</t>
+          <t>Sparq (TL) | AKW Holdings (Term Loan) | AKW Holdings (Common) | Sparq (DDTL) | Sparq (Common Equity)</t>
         </is>
       </c>
       <c r="T55" t="b">
@@ -5075,7 +5093,7 @@
         <v>1</v>
       </c>
       <c r="Q56" t="n">
-        <v>670.9543</v>
+        <v>941.8649</v>
       </c>
       <c r="R56" t="inlineStr">
         <is>
@@ -5159,7 +5177,7 @@
         <v>1</v>
       </c>
       <c r="Q57" t="n">
-        <v>634.9015000000001</v>
+        <v>942.0512</v>
       </c>
       <c r="R57" t="inlineStr">
         <is>
@@ -5227,23 +5245,23 @@
       </c>
       <c r="L58" t="inlineStr">
         <is>
-          <t>Comprehensive Rehab Consultants (Term Loan)</t>
+          <t>Comprehensive Rehab Consultants (Revolver)</t>
         </is>
       </c>
       <c r="M58" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="N58" t="b">
         <v>1</v>
       </c>
       <c r="O58" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="P58" t="n">
         <v>0.9812</v>
       </c>
       <c r="Q58" t="n">
-        <v>310.6171</v>
+        <v>475.5515</v>
       </c>
       <c r="R58" t="inlineStr">
         <is>
@@ -5252,7 +5270,7 @@
       </c>
       <c r="S58" t="inlineStr">
         <is>
-          <t>Comprehensive Rehab Consultants (Term Loan) | Comprehensive Rehab Consultants (Revolver) | Comprehensive Rehab Consultants (Common Equity) | Confluent Health (TL) | Ro Health (Term Loan)</t>
+          <t>Comprehensive Rehab Consultants (Revolver) | Comprehensive Rehab Consultants (Term Loan) | Comprehensive Rehab Consultants (Common Equity) | Ro Health (Revolver) | Nevada Behavioral Health Systems (Revolver)</t>
         </is>
       </c>
       <c r="T58" t="b">
@@ -5327,7 +5345,7 @@
         <v>1</v>
       </c>
       <c r="Q59" t="n">
-        <v>536.6979</v>
+        <v>763.0334</v>
       </c>
       <c r="R59" t="inlineStr">
         <is>
@@ -5411,7 +5429,7 @@
         <v>0.8954</v>
       </c>
       <c r="Q60" t="n">
-        <v>356.2388</v>
+        <v>499.4792</v>
       </c>
       <c r="R60" t="inlineStr">
         <is>
@@ -5495,7 +5513,7 @@
         <v>0.9586</v>
       </c>
       <c r="Q61" t="n">
-        <v>553.5313</v>
+        <v>778.59</v>
       </c>
       <c r="R61" t="inlineStr">
         <is>
@@ -5504,7 +5522,7 @@
       </c>
       <c r="S61" t="inlineStr">
         <is>
-          <t>Evans Network (1L) | Evans Network (2L) | Connatix (Term Loan) | Connatix (Revolver) | Connatix (DDTL)</t>
+          <t>Evans Network (1L) | Evans Network (2L) | Planview (TL) | Rosco (Term Loan) | Connatix (Common Equity)</t>
         </is>
       </c>
       <c r="T61" t="b">
@@ -5579,7 +5597,7 @@
         <v>1</v>
       </c>
       <c r="Q62" t="n">
-        <v>643.9983</v>
+        <v>924.6727</v>
       </c>
       <c r="R62" t="inlineStr">
         <is>
@@ -5647,23 +5665,23 @@
       </c>
       <c r="L63" t="inlineStr">
         <is>
-          <t>Infinity Home Services (Term Loan)</t>
+          <t>Infinity Home Services (Revolver)</t>
         </is>
       </c>
       <c r="M63" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="N63" t="b">
         <v>1</v>
       </c>
       <c r="O63" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="P63" t="n">
         <v>1</v>
       </c>
       <c r="Q63" t="n">
-        <v>461.2423</v>
+        <v>722.9121</v>
       </c>
       <c r="R63" t="inlineStr">
         <is>
@@ -5672,7 +5690,7 @@
       </c>
       <c r="S63" t="inlineStr">
         <is>
-          <t>Infinity Home Services (Term Loan) | Infinity Home Services (Revolver) | Infinity Home Services (Common Equity) | Infinity Home Services (DDTL) | Infinity Home Services (DDTL) CAD</t>
+          <t>Infinity Home Services (Revolver) | Infinity Home Services (Common Equity) | Infinity Home Services (Term Loan) | Infinity Home Services (DDTL) | Infinity Home Services (DDTL) CAD</t>
         </is>
       </c>
       <c r="T63" t="b">
@@ -5747,7 +5765,7 @@
         <v>0.9834000000000001</v>
       </c>
       <c r="Q64" t="n">
-        <v>346.1993</v>
+        <v>484.679</v>
       </c>
       <c r="R64" t="inlineStr">
         <is>
@@ -5831,7 +5849,7 @@
         <v>1</v>
       </c>
       <c r="Q65" t="n">
-        <v>341.2175</v>
+        <v>862.566</v>
       </c>
       <c r="R65" t="inlineStr">
         <is>
@@ -5915,7 +5933,7 @@
         <v>1</v>
       </c>
       <c r="Q66" t="n">
-        <v>224.8001</v>
+        <v>543.4204999999999</v>
       </c>
       <c r="R66" t="inlineStr">
         <is>
@@ -5983,7 +6001,7 @@
       </c>
       <c r="L67" t="inlineStr">
         <is>
-          <t>Any Hour Services (Term Loan)</t>
+          <t>Any Hour Services (Revolver)</t>
         </is>
       </c>
       <c r="M67" t="b">
@@ -5999,7 +6017,7 @@
         <v>1</v>
       </c>
       <c r="Q67" t="n">
-        <v>406.0594</v>
+        <v>991.8898</v>
       </c>
       <c r="R67" t="inlineStr">
         <is>
@@ -6008,7 +6026,7 @@
       </c>
       <c r="S67" t="inlineStr">
         <is>
-          <t>Any Hour Services (Term Loan) | Any Hour Services (Revolver) | Any Hour Services (Common Equity) | Any Hour Services (DDTL) | Any Hour Services (DDTL II)</t>
+          <t>Any Hour Services (Revolver) | Any Hour Services (Term Loan) | Any Hour Services (Common Equity) | Any Hour Services (DDTL) | Any Hour Services (DDTL II)</t>
         </is>
       </c>
       <c r="T67" t="b">
@@ -6067,7 +6085,7 @@
       </c>
       <c r="L68" t="inlineStr">
         <is>
-          <t>Any Hour Services (Term Loan)</t>
+          <t>Any Hour Services (Revolver)</t>
         </is>
       </c>
       <c r="M68" t="b">
@@ -6083,7 +6101,7 @@
         <v>1</v>
       </c>
       <c r="Q68" t="n">
-        <v>406.0594</v>
+        <v>991.8898</v>
       </c>
       <c r="R68" t="inlineStr">
         <is>
@@ -6092,7 +6110,7 @@
       </c>
       <c r="S68" t="inlineStr">
         <is>
-          <t>Any Hour Services (Term Loan) | Any Hour Services (Revolver) | Any Hour Services (Common Equity) | Any Hour Services (DDTL) | Any Hour Services (DDTL II)</t>
+          <t>Any Hour Services (Revolver) | Any Hour Services (Term Loan) | Any Hour Services (Common Equity) | Any Hour Services (DDTL) | Any Hour Services (DDTL II)</t>
         </is>
       </c>
       <c r="T68" t="b">
@@ -6151,23 +6169,23 @@
       </c>
       <c r="L69" t="inlineStr">
         <is>
-          <t>Cano Health (Term Loan)</t>
+          <t>Cano Health (Equity)</t>
         </is>
       </c>
       <c r="M69" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="N69" t="b">
         <v>1</v>
       </c>
       <c r="O69" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="P69" t="n">
         <v>1</v>
       </c>
       <c r="Q69" t="n">
-        <v>317.6277</v>
+        <v>739.448</v>
       </c>
       <c r="R69" t="inlineStr">
         <is>
@@ -6176,7 +6194,7 @@
       </c>
       <c r="S69" t="inlineStr">
         <is>
-          <t>Cano Health (Term Loan) | Cano Health (Equity) | Ro Health (Revolver) | Confluent Health (TL) | Ro Health (Term Loan)</t>
+          <t>Cano Health (Equity) | Cano Health (Term Loan) | Ro Health (Revolver) | Confluent Health (TL) | Ro Health (Term Loan)</t>
         </is>
       </c>
       <c r="T69" t="b">
@@ -6251,7 +6269,7 @@
         <v>1</v>
       </c>
       <c r="Q70" t="n">
-        <v>324.8583</v>
+        <v>814.5942</v>
       </c>
       <c r="R70" t="inlineStr">
         <is>
@@ -6335,7 +6353,7 @@
         <v>1</v>
       </c>
       <c r="Q71" t="n">
-        <v>367.8091</v>
+        <v>945.4287</v>
       </c>
       <c r="R71" t="inlineStr">
         <is>
@@ -6416,10 +6434,10 @@
         <v>3</v>
       </c>
       <c r="P72" t="n">
-        <v>0.9462</v>
+        <v>0.9476</v>
       </c>
       <c r="Q72" t="n">
-        <v>205.575</v>
+        <v>518.7523</v>
       </c>
       <c r="R72" t="inlineStr">
         <is>
@@ -6487,23 +6505,23 @@
       </c>
       <c r="L73" t="inlineStr">
         <is>
-          <t>Recteq (TL)</t>
+          <t>Recteq (Equity)</t>
         </is>
       </c>
       <c r="M73" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="N73" t="b">
         <v>1</v>
       </c>
       <c r="O73" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="P73" t="n">
         <v>1</v>
       </c>
       <c r="Q73" t="n">
-        <v>197.82</v>
+        <v>459.7254</v>
       </c>
       <c r="R73" t="inlineStr">
         <is>
@@ -6512,7 +6530,7 @@
       </c>
       <c r="S73" t="inlineStr">
         <is>
-          <t>Recteq (TL) | Recteq (Equity) | Recteq (Revolver)</t>
+          <t>Recteq (Equity) | Recteq (Revolver) | Recteq (TL)</t>
         </is>
       </c>
       <c r="T73" t="b">
@@ -6587,7 +6605,7 @@
         <v>1</v>
       </c>
       <c r="Q74" t="n">
-        <v>443.6071</v>
+        <v>650.7361</v>
       </c>
       <c r="R74" t="inlineStr">
         <is>
@@ -6671,7 +6689,7 @@
         <v>1</v>
       </c>
       <c r="Q75" t="n">
-        <v>349.183</v>
+        <v>525.0438</v>
       </c>
       <c r="R75" t="inlineStr">
         <is>
@@ -6755,7 +6773,7 @@
         <v>1</v>
       </c>
       <c r="Q76" t="n">
-        <v>506.8933</v>
+        <v>744.9492</v>
       </c>
       <c r="R76" t="inlineStr">
         <is>
@@ -6839,7 +6857,7 @@
         <v>1</v>
       </c>
       <c r="Q77" t="n">
-        <v>420.1781</v>
+        <v>586.803</v>
       </c>
       <c r="R77" t="inlineStr">
         <is>
@@ -6923,7 +6941,7 @@
         <v>1</v>
       </c>
       <c r="Q78" t="n">
-        <v>495.3074</v>
+        <v>694.8678</v>
       </c>
       <c r="R78" t="inlineStr">
         <is>
@@ -7004,10 +7022,10 @@
         <v>3</v>
       </c>
       <c r="P79" t="n">
-        <v>0.7583</v>
+        <v>0.76</v>
       </c>
       <c r="Q79" t="n">
-        <v>581.7938</v>
+        <v>883.1317</v>
       </c>
       <c r="R79" t="inlineStr">
         <is>
@@ -7016,7 +7034,7 @@
       </c>
       <c r="S79" t="inlineStr">
         <is>
-          <t>STG (Second Out Term Loans) | STG (First Out New Money Term Loans) | STG (TL) | BlackHawk Industrial (Incremental TL) | BlackHawk Industrial (TL)</t>
+          <t>STG (Second Out Term Loans) | STG (First Out New Money Term Loans) | STG (TL) | Plimpton &amp; Hills (TL) | Plimpton &amp; Hills (DDTL)</t>
         </is>
       </c>
       <c r="T79" t="b">
@@ -7082,16 +7100,16 @@
         <v>0</v>
       </c>
       <c r="N80" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O80" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="P80" t="n">
         <v>0.9499</v>
       </c>
       <c r="Q80" t="n">
-        <v>273.1139</v>
+        <v>382.3594</v>
       </c>
       <c r="R80" t="inlineStr">
         <is>
@@ -7100,7 +7118,7 @@
       </c>
       <c r="S80" t="inlineStr">
         <is>
-          <t>Sparq (TL) | AKW Holdings (Term Loan) | AKW Holdings (Common) | Sparq (Common Equity) | Sparq (DDTL)</t>
+          <t>Sparq (TL) | AKW Holdings (Term Loan) | AKW Holdings (Common) | Sparq (Revolver) | Sparq (Common Equity)</t>
         </is>
       </c>
       <c r="T80" t="b">
@@ -7175,7 +7193,7 @@
         <v>1</v>
       </c>
       <c r="Q81" t="n">
-        <v>522.6645</v>
+        <v>761.2319</v>
       </c>
       <c r="R81" t="inlineStr">
         <is>
@@ -7184,7 +7202,7 @@
       </c>
       <c r="S81" t="inlineStr">
         <is>
-          <t>Schlesinger (Equity) | Schlesinger (Term Loan) | UniTek (Common Eq) | Premiere Global Services (PGi) (Term Loan) | Premiere Global Services (PGi) (Priority Revolver)</t>
+          <t>Schlesinger (Equity) | Schlesinger (Term Loan) | UniTek (Common Eq) | Schlesinger (Revolver) | Schlesinger (DDTL)</t>
         </is>
       </c>
       <c r="T81" t="b">
@@ -7259,7 +7277,7 @@
         <v>0.9647</v>
       </c>
       <c r="Q82" t="n">
-        <v>310.9658</v>
+        <v>436.6165</v>
       </c>
       <c r="R82" t="inlineStr">
         <is>
@@ -7340,10 +7358,10 @@
         <v>1</v>
       </c>
       <c r="P83" t="n">
-        <v>1.106</v>
+        <v>0.901</v>
       </c>
       <c r="Q83" t="n">
-        <v>323.1901</v>
+        <v>454.638</v>
       </c>
       <c r="R83" t="inlineStr">
         <is>
@@ -7424,10 +7442,10 @@
         <v>1</v>
       </c>
       <c r="P84" t="n">
-        <v>1.2</v>
+        <v>1</v>
       </c>
       <c r="Q84" t="n">
-        <v>686.5144</v>
+        <v>963.2418</v>
       </c>
       <c r="R84" t="inlineStr">
         <is>
@@ -7436,7 +7454,7 @@
       </c>
       <c r="S84" t="inlineStr">
         <is>
-          <t>BiggerPockets (Common Equity) | BiggerPockets (TL) | BiggerPockets (Revolver) | 48Forty (Common Equity) | 48Forty (Term Loan)</t>
+          <t>BiggerPockets (Common Equity) | BiggerPockets (TL) | BiggerPockets (Revolver) | 48Forty (Common Equity) | Harris (Common Equity)</t>
         </is>
       </c>
       <c r="T84" t="b">
@@ -7508,19 +7526,19 @@
         <v>1</v>
       </c>
       <c r="P85" t="n">
-        <v>0.7903</v>
+        <v>0.5929</v>
       </c>
       <c r="Q85" t="n">
-        <v>263.9853</v>
+        <v>389.6323</v>
       </c>
       <c r="R85" t="inlineStr">
         <is>
-          <t>Harris | BioDerm | C5MI | Cascade | Northwinds</t>
+          <t>Harris | BioDerm | C5MI | Cascade | Magnolia</t>
         </is>
       </c>
       <c r="S85" t="inlineStr">
         <is>
-          <t>C5MI (Preferred Equity) | Harris (Preferred Equity) | BioDerm (Preferred Equity) | Cascade (Preferred Equity) | C5MI (Common Equity)</t>
+          <t>C5MI (Preferred Equity) | Harris (Preferred Equity) | BioDerm (Preferred Equity) | Cascade (Preferred Equity) | Magnolia (Preferred Equity)</t>
         </is>
       </c>
       <c r="T85" t="b">
@@ -7592,10 +7610,10 @@
         <v>1</v>
       </c>
       <c r="P86" t="n">
-        <v>1.2</v>
+        <v>1</v>
       </c>
       <c r="Q86" t="n">
-        <v>409.2311</v>
+        <v>605.0894</v>
       </c>
       <c r="R86" t="inlineStr">
         <is>
@@ -7676,10 +7694,10 @@
         <v>1</v>
       </c>
       <c r="P87" t="n">
-        <v>1.2</v>
+        <v>1</v>
       </c>
       <c r="Q87" t="n">
-        <v>345.5332</v>
+        <v>508.5554</v>
       </c>
       <c r="R87" t="inlineStr">
         <is>
@@ -7688,7 +7706,7 @@
       </c>
       <c r="S87" t="inlineStr">
         <is>
-          <t>Connatix (Common Equity) | RTIC (Preferred Equity B) | RTIC (Preferred Equity A) | Vertex (Preferred Equity) | RTIC (Preferred Equity C)</t>
+          <t>Connatix (Common Equity) | Vertex (Preferred Equity) | RTIC (Preferred Equity B) | RTIC (Preferred Equity A) | RTIC (Preferred Equity C)</t>
         </is>
       </c>
       <c r="T87" t="b">
@@ -7760,10 +7778,10 @@
         <v>1</v>
       </c>
       <c r="P88" t="n">
-        <v>1.1831</v>
+        <v>0.9832</v>
       </c>
       <c r="Q88" t="n">
-        <v>337.9748</v>
+        <v>474.6021</v>
       </c>
       <c r="R88" t="inlineStr">
         <is>
@@ -7844,14 +7862,14 @@
         <v>1</v>
       </c>
       <c r="P89" t="n">
-        <v>1.1919</v>
+        <v>0.992</v>
       </c>
       <c r="Q89" t="n">
-        <v>459.7261</v>
+        <v>657.6972</v>
       </c>
       <c r="R89" t="inlineStr">
         <is>
-          <t>Tranzact | 48Forty | Harris | Aechelon | AKW Holdings</t>
+          <t>Tranzact | AKW Holdings | 48Forty | Harris | Aechelon</t>
         </is>
       </c>
       <c r="S89" t="inlineStr">
@@ -7928,14 +7946,14 @@
         <v>1</v>
       </c>
       <c r="P90" t="n">
-        <v>1.0656</v>
+        <v>0.8658</v>
       </c>
       <c r="Q90" t="n">
-        <v>254.6661</v>
+        <v>357.3443</v>
       </c>
       <c r="R90" t="inlineStr">
         <is>
-          <t>Tyto Athene | 48Forty | Harris | Aechelon | AKW Holdings</t>
+          <t>Tyto Athene | AKW Holdings | 48Forty | Harris | Aechelon</t>
         </is>
       </c>
       <c r="S90" t="inlineStr">
@@ -8012,19 +8030,19 @@
         <v>1</v>
       </c>
       <c r="P91" t="n">
-        <v>1.0656</v>
+        <v>0.8658</v>
       </c>
       <c r="Q91" t="n">
-        <v>243.8015</v>
+        <v>341.3221</v>
       </c>
       <c r="R91" t="inlineStr">
         <is>
-          <t>Tyto Athene | Harris | BioDerm | C5MI | AKW Holdings</t>
+          <t>Tyto Athene | AKW Holdings | Harris | BioDerm | C5MI</t>
         </is>
       </c>
       <c r="S91" t="inlineStr">
         <is>
-          <t>Tyto Athene (Pref) | BioDerm (Preferred Equity) | Tyto Athene (Equity) | Harris (Preferred Equity) | C5MI (Preferred Equity)</t>
+          <t>Tyto Athene (Pref) | BioDerm (Preferred Equity) | Harris (Preferred Equity) | Tyto Athene (Equity) | C5MI (Preferred Equity)</t>
         </is>
       </c>
       <c r="T91" t="b">
@@ -8096,10 +8114,10 @@
         <v>1</v>
       </c>
       <c r="P92" t="n">
-        <v>1.1278</v>
+        <v>0.928</v>
       </c>
       <c r="Q92" t="n">
-        <v>344.0517</v>
+        <v>495.753</v>
       </c>
       <c r="R92" t="inlineStr">
         <is>
@@ -8180,10 +8198,10 @@
         <v>1</v>
       </c>
       <c r="P93" t="n">
-        <v>1.1329</v>
+        <v>0.9332</v>
       </c>
       <c r="Q93" t="n">
-        <v>390.6513</v>
+        <v>566.9647</v>
       </c>
       <c r="R93" t="inlineStr">
         <is>
@@ -8232,17 +8250,17 @@
       </c>
       <c r="G94" t="inlineStr">
         <is>
-          <t>Watchtower Holdings</t>
+          <t>Watchtower</t>
         </is>
       </c>
       <c r="H94" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I94" t="b">
         <v>1</v>
       </c>
       <c r="J94" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K94" t="inlineStr">
         <is>
@@ -8264,19 +8282,19 @@
         <v>1</v>
       </c>
       <c r="P94" t="n">
-        <v>1.1889</v>
+        <v>1</v>
       </c>
       <c r="Q94" t="n">
-        <v>333.6397</v>
+        <v>495.1412</v>
       </c>
       <c r="R94" t="inlineStr">
         <is>
-          <t>Watchtower Holdings | Watchtower | Watchtower Buyer | 48Forty | AKW Holdings</t>
+          <t>Watchtower | Watchtower Holdings | Watchtower Buyer | AKW Holdings | 48Forty</t>
         </is>
       </c>
       <c r="S94" t="inlineStr">
         <is>
-          <t>Watchtower Holding (Common Equity) | AKW Holdings (Common) | 48Forty (Common Equity) | 48Forty (Term Loan) | AKW Holdings (Term Loan)</t>
+          <t>Watchtower Holding (Common Equity) | AKW Holdings (Common) | 48Forty (Common Equity) | Watchtower (TL) | Watchtower (Revolver)</t>
         </is>
       </c>
       <c r="T94" t="b">
@@ -8348,14 +8366,14 @@
         <v>1</v>
       </c>
       <c r="P95" t="n">
-        <v>1.2</v>
+        <v>1</v>
       </c>
       <c r="Q95" t="n">
-        <v>471.985</v>
+        <v>690.3403</v>
       </c>
       <c r="R95" t="inlineStr">
         <is>
-          <t>Watterson | 48Forty | Harris | Aechelon | AKW Holdings</t>
+          <t>Watterson | AKW Holdings | 48Forty | Harris | Aechelon</t>
         </is>
       </c>
       <c r="S95" t="inlineStr">
@@ -8496,14 +8514,14 @@
         </is>
       </c>
       <c r="L2" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="M2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="N2" t="inlineStr">
         <is>
-          <t>88.9%</t>
+          <t>100.0%</t>
         </is>
       </c>
     </row>
@@ -8517,14 +8535,14 @@
         <v>13</v>
       </c>
       <c r="C3" t="n">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="D3" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>92.3%</t>
+          <t>84.6%</t>
         </is>
       </c>
       <c r="F3" t="n">
@@ -8593,14 +8611,14 @@
         </is>
       </c>
       <c r="I4" t="n">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="J4" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="K4" t="inlineStr">
         <is>
-          <t>78.6%</t>
+          <t>92.9%</t>
         </is>
       </c>
       <c r="L4" t="n">
@@ -8647,14 +8665,14 @@
         </is>
       </c>
       <c r="I5" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="J5" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="K5" t="inlineStr">
         <is>
-          <t>11.1%</t>
+          <t>33.3%</t>
         </is>
       </c>
       <c r="L5" t="n">
@@ -8679,14 +8697,14 @@
         <v>31</v>
       </c>
       <c r="C6" t="n">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="D6" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>87.1%</t>
+          <t>90.3%</t>
         </is>
       </c>
       <c r="F6" t="n">
@@ -8701,25 +8719,25 @@
         </is>
       </c>
       <c r="I6" t="n">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="J6" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="K6" t="inlineStr">
         <is>
-          <t>74.2%</t>
+          <t>80.6%</t>
         </is>
       </c>
       <c r="L6" t="n">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="M6" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="N6" t="inlineStr">
         <is>
-          <t>80.6%</t>
+          <t>87.1%</t>
         </is>
       </c>
     </row>
@@ -8755,14 +8773,14 @@
         </is>
       </c>
       <c r="I7" t="n">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="J7" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="K7" t="inlineStr">
         <is>
-          <t>61.1%</t>
+          <t>55.6%</t>
         </is>
       </c>
       <c r="L7" t="n">

</xml_diff>

<commit_message>
Push for entire retrieval including master and mapped
</commit_message>
<xml_diff>
--- a/evaluation_results.xlsx
+++ b/evaluation_results.xlsx
@@ -1172,19 +1172,19 @@
         <v>1</v>
       </c>
       <c r="P9" t="n">
-        <v>0.9023</v>
+        <v>1</v>
       </c>
       <c r="Q9" t="n">
-        <v>605.7479</v>
+        <v>1</v>
       </c>
       <c r="R9" t="inlineStr">
         <is>
-          <t>Bland Landscaping | Watchtower Holdings</t>
+          <t>Bland Landscaping</t>
         </is>
       </c>
       <c r="S9" t="inlineStr">
         <is>
-          <t>Bland Landscaping (DDTL) | Bland Landscaping (Term Loan) | Bland Landscaping (Revolver) | Watchtower Holding (Common Equity)</t>
+          <t>Bland Landscaping (DDTL)</t>
         </is>
       </c>
       <c r="T9" t="b">
@@ -1599,12 +1599,12 @@
       </c>
       <c r="R14" t="inlineStr">
         <is>
-          <t>Centauri Health | Watchtower Buyer | APHIX | Carisk Partners | Connatix</t>
+          <t>Centauri Health | Watchtower Buyer | 360DG | Integrated Data Services | Tranzact</t>
         </is>
       </c>
       <c r="S14" t="inlineStr">
         <is>
-          <t>Centauri Health (TL) | Centauri Health (Revolver) | Watchtower Buyer (Revolver) | Centauri Health (DDTL) | Carisk Partners (Revolver)</t>
+          <t>Centauri Health (TL) | Centauri Health (Revolver) | Watchtower Buyer (Revolver) | Centauri Health (DDTL) | 360DG (Revolver)</t>
         </is>
       </c>
       <c r="T14" t="b">
@@ -2264,14 +2264,14 @@
         <v>5</v>
       </c>
       <c r="P22" t="n">
-        <v>0.8549</v>
+        <v>0.8537</v>
       </c>
       <c r="Q22" t="n">
-        <v>85.36020000000001</v>
+        <v>86.6747</v>
       </c>
       <c r="R22" t="inlineStr">
         <is>
-          <t>OSG Billing Services | U.S. Well | ImagineAcquisitionCo | AKW Holdings | None</t>
+          <t>OSG Billing Services | U.S. Well | ImagineAcquisitionCo | None | AKW Holdings</t>
         </is>
       </c>
       <c r="S22" t="inlineStr">
@@ -2758,10 +2758,10 @@
       </c>
       <c r="O28" t="inlineStr"/>
       <c r="P28" t="n">
-        <v>0.6002999999999999</v>
+        <v>0.5628</v>
       </c>
       <c r="Q28" t="n">
-        <v>36.3303</v>
+        <v>36.6381</v>
       </c>
       <c r="R28" t="inlineStr">
         <is>
@@ -2925,7 +2925,7 @@
         <v>1</v>
       </c>
       <c r="Q30" t="n">
-        <v>432.755</v>
+        <v>435.0036</v>
       </c>
       <c r="R30" t="inlineStr">
         <is>
@@ -2934,7 +2934,7 @@
       </c>
       <c r="S30" t="inlineStr">
         <is>
-          <t>PlayPower (Term Loan)</t>
+          <t>PlayPower (Term Loan) | Bluebird (Term Loan) | BlueHalo (Term Loan) | Aechelon (Term Loan) | 360DG (Term Loan)</t>
         </is>
       </c>
       <c r="T30" t="b">
@@ -3087,13 +3087,13 @@
         <v>0</v>
       </c>
       <c r="O32" t="n">
-        <v>10</v>
+        <v>15</v>
       </c>
       <c r="P32" t="n">
         <v>0.7469</v>
       </c>
       <c r="Q32" t="n">
-        <v>391.6117</v>
+        <v>396.0039</v>
       </c>
       <c r="R32" t="inlineStr">
         <is>
@@ -3102,7 +3102,7 @@
       </c>
       <c r="S32" t="inlineStr">
         <is>
-          <t>APT Healthcare (Incr. DDTL) | Zips (DDTL) | APT Healthcare (Term Loan) | Lilly Lashes (TL) | APT Healthcare (Common Equity)</t>
+          <t>APT Healthcare (Incr. DDTL) | Zips (DDTL) | Bland Landscaping (DDTL) | AFC Industries (DDTL) | Carnegie Dartlet (DDTL)</t>
         </is>
       </c>
       <c r="T32" t="b">
@@ -3170,10 +3170,10 @@
       </c>
       <c r="O33" t="inlineStr"/>
       <c r="P33" t="n">
-        <v>0.8365</v>
+        <v>0.8363</v>
       </c>
       <c r="Q33" t="n">
-        <v>394.7907</v>
+        <v>399.9936</v>
       </c>
       <c r="R33" t="inlineStr">
         <is>
@@ -3254,19 +3254,19 @@
         <v>1</v>
       </c>
       <c r="P34" t="n">
-        <v>0.9995000000000001</v>
+        <v>1</v>
       </c>
       <c r="Q34" t="n">
-        <v>618.7388999999999</v>
+        <v>1</v>
       </c>
       <c r="R34" t="inlineStr">
         <is>
-          <t>48Forty | Smartronix / Trident | Altamira | Douglas | Engine &amp; Transmission Exchange</t>
+          <t>48Forty</t>
         </is>
       </c>
       <c r="S34" t="inlineStr">
         <is>
-          <t>48Forty (Common Equity) | 48Forty (Term Loan) | Altamira (Common Equity) | Smartronix / Trident (Common Equity) | Engine &amp; Transmission Exchange (Common Equity)</t>
+          <t>48Forty (Common Equity)</t>
         </is>
       </c>
       <c r="T34" t="b">
@@ -3338,19 +3338,19 @@
         <v>1</v>
       </c>
       <c r="P35" t="n">
-        <v>0.9834000000000001</v>
+        <v>1</v>
       </c>
       <c r="Q35" t="n">
-        <v>537.6147</v>
+        <v>1</v>
       </c>
       <c r="R35" t="inlineStr">
         <is>
-          <t>4Wall Entertainment | AKW Holdings</t>
+          <t>4Wall Entertainment</t>
         </is>
       </c>
       <c r="S35" t="inlineStr">
         <is>
-          <t>4Wall Entertainment (Term Loan) | 4Wall Entertainment (DDTL) | 4Wall Entertainment (Revolver) | AKW Holdings (Term Loan) | AKW Holdings (Common)</t>
+          <t>4Wall Entertainment (Term Loan)</t>
         </is>
       </c>
       <c r="T35" t="b">
@@ -3425,16 +3425,16 @@
         <v>1</v>
       </c>
       <c r="Q36" t="n">
-        <v>706.376</v>
+        <v>1</v>
       </c>
       <c r="R36" t="inlineStr">
         <is>
-          <t>BBB Industries | STG Logistics | Adweek | Aspect Software | Health-E Commerce</t>
+          <t>BBB Industries</t>
         </is>
       </c>
       <c r="S36" t="inlineStr">
         <is>
-          <t>BBB Industries (First Lien Term Loan) | BBB Industries (Second Lien Term Loan) | STG (TL) | Adweek (Term Loan) | Adweek (DDTL)</t>
+          <t>BBB Industries (First Lien Term Loan)</t>
         </is>
       </c>
       <c r="T36" t="b">
@@ -3509,16 +3509,16 @@
         <v>1</v>
       </c>
       <c r="Q37" t="n">
-        <v>658.7212</v>
+        <v>1</v>
       </c>
       <c r="R37" t="inlineStr">
         <is>
-          <t>Big Top Manufacturing | None | AKW Holdings</t>
+          <t>Big Top Manufacturing</t>
         </is>
       </c>
       <c r="S37" t="inlineStr">
         <is>
-          <t>Big Top Manufacturing (Term Loan) | Big Top Manufacturing (Revolver) | Big Top Manufacturing (Common Equity) | AKW Holdings (Term Loan) | IMIA (Term Loan)</t>
+          <t>Big Top Manufacturing (Term Loan)</t>
         </is>
       </c>
       <c r="T37" t="b">
@@ -3558,17 +3558,17 @@
       </c>
       <c r="G38" t="inlineStr">
         <is>
-          <t>Global</t>
+          <t>BlueHalo</t>
         </is>
       </c>
       <c r="H38" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I38" t="b">
         <v>1</v>
       </c>
       <c r="J38" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K38" t="inlineStr">
         <is>
@@ -3577,32 +3577,32 @@
       </c>
       <c r="L38" t="inlineStr">
         <is>
-          <t>Global (Term Loan)</t>
+          <t>BlueHalo (Term Loan)</t>
         </is>
       </c>
       <c r="M38" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="N38" t="b">
         <v>1</v>
       </c>
       <c r="O38" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="P38" t="n">
-        <v>0.8559</v>
+        <v>1</v>
       </c>
       <c r="Q38" t="n">
-        <v>374.5238</v>
+        <v>1</v>
       </c>
       <c r="R38" t="inlineStr">
         <is>
-          <t>Global | BlueHalo | Insight Global | Schlesinger | UniTek</t>
+          <t>BlueHalo</t>
         </is>
       </c>
       <c r="S38" t="inlineStr">
         <is>
-          <t>Global (Term Loan) | BlueHalo (Term Loan) | Insight Global (TL) | Schlesinger (Term Loan) | Schlesinger (DDTL)</t>
+          <t>BlueHalo (Term Loan)</t>
         </is>
       </c>
       <c r="T38" t="b">
@@ -3677,16 +3677,16 @@
         <v>1</v>
       </c>
       <c r="Q39" t="n">
-        <v>571.072</v>
+        <v>1</v>
       </c>
       <c r="R39" t="inlineStr">
         <is>
-          <t>Integrated Data Services | Watchtower Buyer | nThrive | Big Top Manufacturing | APHIX</t>
+          <t>Integrated Data Services</t>
         </is>
       </c>
       <c r="S39" t="inlineStr">
         <is>
-          <t>Integrated Data Services (TL) | Integrated Data Services (Rev) | Watchtower Buyer (TL) | Watchtower Buyer (DDTL) | Aphix (Term Loan)</t>
+          <t>Integrated Data Services (TL)</t>
         </is>
       </c>
       <c r="T39" t="b">
@@ -3758,19 +3758,19 @@
         <v>1</v>
       </c>
       <c r="P40" t="n">
-        <v>0.9758</v>
+        <v>1</v>
       </c>
       <c r="Q40" t="n">
-        <v>458.7628</v>
+        <v>1</v>
       </c>
       <c r="R40" t="inlineStr">
         <is>
-          <t>KNS | STG Logistics | Adweek | Aspect Software | Health-E Commerce</t>
+          <t>KNS</t>
         </is>
       </c>
       <c r="S40" t="inlineStr">
         <is>
-          <t>KNS (Term Loan) | STG (TL) | Adweek (Term Loan) | Adweek (DDTL) | Health-E Commerce (Term Loan)</t>
+          <t>KNS (Term Loan)</t>
         </is>
       </c>
       <c r="T40" t="b">
@@ -3845,16 +3845,16 @@
         <v>1</v>
       </c>
       <c r="Q41" t="n">
-        <v>649.8196</v>
+        <v>1</v>
       </c>
       <c r="R41" t="inlineStr">
         <is>
-          <t>Radius Aerospace | Cadence Aerospace | MAG Aerospace</t>
+          <t>Radius Aerospace</t>
         </is>
       </c>
       <c r="S41" t="inlineStr">
         <is>
-          <t>Radius Aerospace (Term Loan) | Radius Aerospace (Revolver) | MAG Aerospace (TL) | Cadence Aerospace</t>
+          <t>Radius Aerospace (Term Loan)</t>
         </is>
       </c>
       <c r="T41" t="b">
@@ -3929,7 +3929,7 @@
         <v>1</v>
       </c>
       <c r="Q42" t="n">
-        <v>538.772</v>
+        <v>1</v>
       </c>
       <c r="R42" t="inlineStr">
         <is>
@@ -3938,7 +3938,7 @@
       </c>
       <c r="S42" t="inlineStr">
         <is>
-          <t>Roofed Right America (Term Loan) | Roofed Right America (DDTL 2) | Roofed Right America (DDTL 1) | Roofed Right America (Revolver)</t>
+          <t>Roofed Right America (Term Loan)</t>
         </is>
       </c>
       <c r="T42" t="b">
@@ -4009,7 +4009,7 @@
         <v>0.7544</v>
       </c>
       <c r="Q43" t="n">
-        <v>391.6918</v>
+        <v>396.3347</v>
       </c>
       <c r="R43" t="inlineStr">
         <is>
@@ -4018,7 +4018,7 @@
       </c>
       <c r="S43" t="inlineStr">
         <is>
-          <t>US Fertility (DDTL) | TVC (DDTL) | TVC (TL) | US Fertility (Term Loan) | TVC (Revolver)</t>
+          <t>US Fertility (DDTL) | TVC (DDTL) | TVC (TL) | US Fertility (Term Loan) | Bland Landscaping (DDTL)</t>
         </is>
       </c>
       <c r="T43" t="b">
@@ -4089,7 +4089,7 @@
         <v>0.7544</v>
       </c>
       <c r="Q44" t="n">
-        <v>292.8177</v>
+        <v>294.2774</v>
       </c>
       <c r="R44" t="inlineStr">
         <is>
@@ -4098,7 +4098,7 @@
       </c>
       <c r="S44" t="inlineStr">
         <is>
-          <t>TVC (TL) | US Fertility (Term Loan) | US Fertility (DDTL) | TVC (DDTL) | TVC (Revolver)</t>
+          <t>TVC (TL) | US Fertility (Term Loan) | US Fertility (DDTL) | TVC (DDTL) | MeritDirect (Term Loan)</t>
         </is>
       </c>
       <c r="T44" t="b">
@@ -4173,7 +4173,7 @@
         <v>0.999</v>
       </c>
       <c r="Q45" t="n">
-        <v>590.5582000000001</v>
+        <v>591.8692</v>
       </c>
       <c r="R45" t="inlineStr">
         <is>
@@ -4182,7 +4182,7 @@
       </c>
       <c r="S45" t="inlineStr">
         <is>
-          <t>Aeronix (DDTL) | Aeronix (Common Equity) | AKW Holdings (Term Loan) | Aeronix (TL) | AKW Holdings (Common)</t>
+          <t>Aeronix (DDTL) | Aeronix (Common Equity) | AKW Holdings (Term Loan) | Aeronix (TL) | 4Wall Entertainment (Term Loan)</t>
         </is>
       </c>
       <c r="T45" t="b">
@@ -4254,19 +4254,19 @@
         <v>1</v>
       </c>
       <c r="P46" t="n">
-        <v>0.8377</v>
+        <v>1</v>
       </c>
       <c r="Q46" t="n">
-        <v>488.6119</v>
+        <v>1</v>
       </c>
       <c r="R46" t="inlineStr">
         <is>
-          <t>Dr. Scholl's | Apex Service Partners | API Technologies | Wheel Pros | Paris Presents</t>
+          <t>Dr. Scholl's</t>
         </is>
       </c>
       <c r="S46" t="inlineStr">
         <is>
-          <t>Dr. Scholl's (Term Loan) | Dr. Scholl's (Revolver) | API Technologies (TL) | Apex (DDTL III) | Wheel Pros (1L)</t>
+          <t>Dr. Scholl's (Term Loan)</t>
         </is>
       </c>
       <c r="T46" t="b">
@@ -4338,19 +4338,19 @@
         <v>1</v>
       </c>
       <c r="P47" t="n">
-        <v>0.8461</v>
+        <v>1</v>
       </c>
       <c r="Q47" t="n">
-        <v>583.1864</v>
+        <v>1</v>
       </c>
       <c r="R47" t="inlineStr">
         <is>
-          <t>MCR | Sabel Systems | Signature Systems Group | Nevada Behavioral Health Systems | None</t>
+          <t>MCR</t>
         </is>
       </c>
       <c r="S47" t="inlineStr">
         <is>
-          <t>MCR (Term Loan) | MCR (Revolver) | Kentucky Downs (DDTL A) | FlexPrint (DDTL) | Research Horizons (DDTL)</t>
+          <t>MCR (Term Loan)</t>
         </is>
       </c>
       <c r="T47" t="b">
@@ -4418,10 +4418,10 @@
       </c>
       <c r="O48" t="inlineStr"/>
       <c r="P48" t="n">
-        <v>0.5482</v>
+        <v>0.5505</v>
       </c>
       <c r="Q48" t="n">
-        <v>233.9925</v>
+        <v>235.981</v>
       </c>
       <c r="R48" t="inlineStr">
         <is>
@@ -4484,7 +4484,7 @@
       </c>
       <c r="K49" t="inlineStr">
         <is>
-          <t>STG (TL)</t>
+          <t>STG (First Out New Money Term Loans)</t>
         </is>
       </c>
       <c r="L49" t="inlineStr">
@@ -4493,28 +4493,28 @@
         </is>
       </c>
       <c r="M49" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="N49" t="b">
         <v>1</v>
       </c>
       <c r="O49" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="P49" t="n">
-        <v>0.76</v>
+        <v>1</v>
       </c>
       <c r="Q49" t="n">
-        <v>887.1277</v>
+        <v>1</v>
       </c>
       <c r="R49" t="inlineStr">
         <is>
-          <t>STG Logistics | Plimpton &amp; Hills | BlackHawk Industrial | WhiteHawk Industrial</t>
+          <t>STG Logistics</t>
         </is>
       </c>
       <c r="S49" t="inlineStr">
         <is>
-          <t>STG (First Out New Money Term Loans) | STG (Second Out Term Loans) | STG (TL) | Plimpton &amp; Hills (TL) | Plimpton &amp; Hills (DDTL)</t>
+          <t>STG (First Out New Money Term Loans)</t>
         </is>
       </c>
       <c r="T49" t="b">
@@ -4589,7 +4589,7 @@
         <v>1</v>
       </c>
       <c r="Q50" t="n">
-        <v>667.8467000000001</v>
+        <v>672.4636</v>
       </c>
       <c r="R50" t="inlineStr">
         <is>
@@ -4670,19 +4670,19 @@
         <v>1</v>
       </c>
       <c r="P51" t="n">
-        <v>0.9834000000000001</v>
+        <v>1</v>
       </c>
       <c r="Q51" t="n">
-        <v>537.6147</v>
+        <v>1</v>
       </c>
       <c r="R51" t="inlineStr">
         <is>
-          <t>4Wall Entertainment | AKW Holdings</t>
+          <t>4Wall Entertainment</t>
         </is>
       </c>
       <c r="S51" t="inlineStr">
         <is>
-          <t>4Wall Entertainment (Term Loan) | 4Wall Entertainment (DDTL) | 4Wall Entertainment (Revolver) | AKW Holdings (Term Loan) | AKW Holdings (Common)</t>
+          <t>4Wall Entertainment (Term Loan)</t>
         </is>
       </c>
       <c r="T51" t="b">
@@ -4757,16 +4757,16 @@
         <v>1</v>
       </c>
       <c r="Q52" t="n">
-        <v>688.3133</v>
+        <v>1</v>
       </c>
       <c r="R52" t="inlineStr">
         <is>
-          <t>A1 Garage | A2 Garge | None | Guild Garage Group | Omnia</t>
+          <t>A1 Garage</t>
         </is>
       </c>
       <c r="S52" t="inlineStr">
         <is>
-          <t>A1 Garage (Common Equity) | A1 Garage (Revolver) | A1 Garage (Term Loan) | A1 Garage (DDTL) | Guild Garage Group (Common Equity)</t>
+          <t>A1 Garage (Common Equity)</t>
         </is>
       </c>
       <c r="T52" t="b">
@@ -4841,7 +4841,7 @@
         <v>1</v>
       </c>
       <c r="Q53" t="n">
-        <v>709.112</v>
+        <v>1</v>
       </c>
       <c r="R53" t="inlineStr">
         <is>
@@ -4850,7 +4850,7 @@
       </c>
       <c r="S53" t="inlineStr">
         <is>
-          <t>Archer Lewis (Revolver) | Archer Lewis (Term Loan) | Archer Lewis (Unfunded DDTL B) | Archer Lewis (Unfunded DDTL A) | Archer Lewis (Common Equity)</t>
+          <t>Archer Lewis (Revolver)</t>
         </is>
       </c>
       <c r="T53" t="b">
@@ -4925,16 +4925,16 @@
         <v>1</v>
       </c>
       <c r="Q54" t="n">
-        <v>820.9715</v>
+        <v>1</v>
       </c>
       <c r="R54" t="inlineStr">
         <is>
-          <t>Beta+ | API Technologies | Altamira | Nuvei | Lynx Technologies</t>
+          <t>Beta+</t>
         </is>
       </c>
       <c r="S54" t="inlineStr">
         <is>
-          <t>Beta+ (TL) | API Technologies (TL) | Lynx Technologies (TL) | Altamira (TL) | Nuvei (Term Loan)</t>
+          <t>Beta+ (TL)</t>
         </is>
       </c>
       <c r="T54" t="b">
@@ -5006,19 +5006,19 @@
         <v>1</v>
       </c>
       <c r="P55" t="n">
-        <v>0.9499</v>
+        <v>1</v>
       </c>
       <c r="Q55" t="n">
-        <v>411.894</v>
+        <v>1</v>
       </c>
       <c r="R55" t="inlineStr">
         <is>
-          <t>Sparq | AKW Holdings</t>
+          <t>Sparq</t>
         </is>
       </c>
       <c r="S55" t="inlineStr">
         <is>
-          <t>Sparq (TL) | AKW Holdings (Term Loan) | AKW Holdings (Common) | Sparq (DDTL) | Sparq (Common Equity)</t>
+          <t>Sparq (TL)</t>
         </is>
       </c>
       <c r="T55" t="b">
@@ -5093,7 +5093,7 @@
         <v>1</v>
       </c>
       <c r="Q56" t="n">
-        <v>941.8649</v>
+        <v>1</v>
       </c>
       <c r="R56" t="inlineStr">
         <is>
@@ -5102,7 +5102,7 @@
       </c>
       <c r="S56" t="inlineStr">
         <is>
-          <t>BiggerPockets (Revolver) | BiggerPockets (TL) | BiggerPockets (Common Equity)</t>
+          <t>BiggerPockets (Revolver)</t>
         </is>
       </c>
       <c r="T56" t="b">
@@ -5177,7 +5177,7 @@
         <v>1</v>
       </c>
       <c r="Q57" t="n">
-        <v>942.0512</v>
+        <v>1</v>
       </c>
       <c r="R57" t="inlineStr">
         <is>
@@ -5186,7 +5186,7 @@
       </c>
       <c r="S57" t="inlineStr">
         <is>
-          <t>Carnegie Dartlet (DDTL) | Carnegie Dartlet (Term Loan) | Carnegie Dartlet (Revolver) | Carnegie Dartlet (Common Equity)</t>
+          <t>Carnegie Dartlet (DDTL)</t>
         </is>
       </c>
       <c r="T57" t="b">
@@ -5258,19 +5258,19 @@
         <v>1</v>
       </c>
       <c r="P58" t="n">
-        <v>0.9812</v>
+        <v>1</v>
       </c>
       <c r="Q58" t="n">
-        <v>475.5515</v>
+        <v>1</v>
       </c>
       <c r="R58" t="inlineStr">
         <is>
-          <t>Comprehensive Rehab Consultants | Ro Health | Confluent Health | Cano Health | Nevada Behavioral Health Systems</t>
+          <t>Comprehensive Rehab Consultants</t>
         </is>
       </c>
       <c r="S58" t="inlineStr">
         <is>
-          <t>Comprehensive Rehab Consultants (Revolver) | Comprehensive Rehab Consultants (Term Loan) | Comprehensive Rehab Consultants (Common Equity) | Ro Health (Revolver) | Nevada Behavioral Health Systems (Revolver)</t>
+          <t>Comprehensive Rehab Consultants (Revolver)</t>
         </is>
       </c>
       <c r="T58" t="b">
@@ -5345,16 +5345,16 @@
         <v>1</v>
       </c>
       <c r="Q59" t="n">
-        <v>763.0334</v>
+        <v>1</v>
       </c>
       <c r="R59" t="inlineStr">
         <is>
-          <t>Engine &amp; Transmission Exchange | Infosoft | Lilly Lashes | Loving Tan | Schlesinger</t>
+          <t>Engine &amp; Transmission Exchange</t>
         </is>
       </c>
       <c r="S59" t="inlineStr">
         <is>
-          <t>Engine &amp; Transmission Exchange (Common Equity) | Engine &amp; Transmission Exchange (Promissory Note) | Infosoft (Common Equity) | Schlesinger (Equity) | Lilly Lashes (Equity)</t>
+          <t>Engine &amp; Transmission Exchange (Common Equity)</t>
         </is>
       </c>
       <c r="T59" t="b">
@@ -5426,19 +5426,19 @@
         <v>1</v>
       </c>
       <c r="P60" t="n">
-        <v>0.8954</v>
+        <v>1</v>
       </c>
       <c r="Q60" t="n">
-        <v>499.4792</v>
+        <v>1</v>
       </c>
       <c r="R60" t="inlineStr">
         <is>
-          <t>Epiq | ImagineAcquisitionCo</t>
+          <t>Epiq</t>
         </is>
       </c>
       <c r="S60" t="inlineStr">
         <is>
-          <t>Epiq (Common) | Imagine Topco. L.P. (Common Equity - Series B) | Imagine Topco. L.P. (Preferred Equity - Series A) | Epiq (TL) | Epiq (Revolver)</t>
+          <t>Epiq (Common)</t>
         </is>
       </c>
       <c r="T60" t="b">
@@ -5510,19 +5510,19 @@
         <v>1</v>
       </c>
       <c r="P61" t="n">
-        <v>0.9586</v>
+        <v>1</v>
       </c>
       <c r="Q61" t="n">
-        <v>778.59</v>
+        <v>1</v>
       </c>
       <c r="R61" t="inlineStr">
         <is>
-          <t>Evans Network | Connatix | Planview | Rancho Medical | Rosco</t>
+          <t>Evans Network</t>
         </is>
       </c>
       <c r="S61" t="inlineStr">
         <is>
-          <t>Evans Network (1L) | Evans Network (2L) | Planview (TL) | Rosco (Term Loan) | Connatix (Common Equity)</t>
+          <t>Evans Network (1L)</t>
         </is>
       </c>
       <c r="T61" t="b">
@@ -5597,16 +5597,16 @@
         <v>1</v>
       </c>
       <c r="Q62" t="n">
-        <v>924.6727</v>
+        <v>1</v>
       </c>
       <c r="R62" t="inlineStr">
         <is>
-          <t>Federal Advisory Partners | None | First Medical Associates</t>
+          <t>Federal Advisory Partners</t>
         </is>
       </c>
       <c r="S62" t="inlineStr">
         <is>
-          <t>Federal Advisory Partners (First Lien Term Loan) | Federal Advisory Partners (Term Loan) | Federal Advisory Partners (Revolver) | First Medical Associates (Term Loan) | First Medical Associates (DDTL)</t>
+          <t>Federal Advisory Partners (First Lien Term Loan)</t>
         </is>
       </c>
       <c r="T62" t="b">
@@ -5681,16 +5681,16 @@
         <v>1</v>
       </c>
       <c r="Q63" t="n">
-        <v>722.9121</v>
+        <v>1</v>
       </c>
       <c r="R63" t="inlineStr">
         <is>
-          <t>Infinity Home Services | United Land Services | Any Hour Services | Applied Technical Services | IDC Infusion Services</t>
+          <t>Infinity Home Services</t>
         </is>
       </c>
       <c r="S63" t="inlineStr">
         <is>
-          <t>Infinity Home Services (Revolver) | Infinity Home Services (Common Equity) | Infinity Home Services (Term Loan) | Infinity Home Services (DDTL) | Infinity Home Services (DDTL) CAD</t>
+          <t>Infinity Home Services (Revolver)</t>
         </is>
       </c>
       <c r="T63" t="b">
@@ -5849,7 +5849,7 @@
         <v>1</v>
       </c>
       <c r="Q65" t="n">
-        <v>862.566</v>
+        <v>873.5107</v>
       </c>
       <c r="R65" t="inlineStr">
         <is>
@@ -5933,7 +5933,7 @@
         <v>1</v>
       </c>
       <c r="Q66" t="n">
-        <v>543.4204999999999</v>
+        <v>546.4172</v>
       </c>
       <c r="R66" t="inlineStr">
         <is>
@@ -6017,7 +6017,7 @@
         <v>1</v>
       </c>
       <c r="Q67" t="n">
-        <v>991.8898</v>
+        <v>1005.7311</v>
       </c>
       <c r="R67" t="inlineStr">
         <is>
@@ -6101,7 +6101,7 @@
         <v>1</v>
       </c>
       <c r="Q68" t="n">
-        <v>991.8898</v>
+        <v>1005.7311</v>
       </c>
       <c r="R68" t="inlineStr">
         <is>
@@ -6185,7 +6185,7 @@
         <v>1</v>
       </c>
       <c r="Q69" t="n">
-        <v>739.448</v>
+        <v>746.6063</v>
       </c>
       <c r="R69" t="inlineStr">
         <is>
@@ -6269,16 +6269,16 @@
         <v>1</v>
       </c>
       <c r="Q70" t="n">
-        <v>814.5942</v>
+        <v>1</v>
       </c>
       <c r="R70" t="inlineStr">
         <is>
-          <t>Dr. Scholl's | Dr. Squatch</t>
+          <t>Dr. Scholl's</t>
         </is>
       </c>
       <c r="S70" t="inlineStr">
         <is>
-          <t>Dr. Scholl's (Revolver) | Dr. Scholl's (Term Loan) | Dr. Squatch (Term Loan) | Dr. Squatch (Revolver) | Dr. Squatch (DDTL)</t>
+          <t>Dr. Scholl's (Revolver)</t>
         </is>
       </c>
       <c r="T70" t="b">
@@ -6353,7 +6353,7 @@
         <v>1</v>
       </c>
       <c r="Q71" t="n">
-        <v>945.4287</v>
+        <v>949.814</v>
       </c>
       <c r="R71" t="inlineStr">
         <is>
@@ -6434,10 +6434,10 @@
         <v>3</v>
       </c>
       <c r="P72" t="n">
-        <v>0.9476</v>
+        <v>0.9471000000000001</v>
       </c>
       <c r="Q72" t="n">
-        <v>518.7523</v>
+        <v>524.371</v>
       </c>
       <c r="R72" t="inlineStr">
         <is>
@@ -6521,7 +6521,7 @@
         <v>1</v>
       </c>
       <c r="Q73" t="n">
-        <v>459.7254</v>
+        <v>1</v>
       </c>
       <c r="R73" t="inlineStr">
         <is>
@@ -6530,7 +6530,7 @@
       </c>
       <c r="S73" t="inlineStr">
         <is>
-          <t>Recteq (Equity) | Recteq (Revolver) | Recteq (TL)</t>
+          <t>Recteq (Equity)</t>
         </is>
       </c>
       <c r="T73" t="b">
@@ -6605,16 +6605,16 @@
         <v>1</v>
       </c>
       <c r="Q74" t="n">
-        <v>650.7361</v>
+        <v>1</v>
       </c>
       <c r="R74" t="inlineStr">
         <is>
-          <t>Watterson | AKW Holdings</t>
+          <t>Watterson</t>
         </is>
       </c>
       <c r="S74" t="inlineStr">
         <is>
-          <t>Watterson (Revolver) | Watterson (TL) | Watterson (Equity) | Watterson (DDTL) | AKW Holdings (Term Loan)</t>
+          <t>Watterson (Revolver)</t>
         </is>
       </c>
       <c r="T74" t="b">
@@ -6689,16 +6689,16 @@
         <v>1</v>
       </c>
       <c r="Q75" t="n">
-        <v>525.0438</v>
+        <v>1</v>
       </c>
       <c r="R75" t="inlineStr">
         <is>
-          <t>Watchtower Buyer | Watchtower | Watchtower Holdings | APHIX | Carisk Partners</t>
+          <t>Watchtower Buyer</t>
         </is>
       </c>
       <c r="S75" t="inlineStr">
         <is>
-          <t>Watchtower Buyer (Revolver) | Watchtower Buyer (TL) | Watchtower Buyer (DDTL) | Watchtower (Revolver) | Carisk Partners (Revolver)</t>
+          <t>Watchtower Buyer (Revolver)</t>
         </is>
       </c>
       <c r="T75" t="b">
@@ -6773,7 +6773,7 @@
         <v>1</v>
       </c>
       <c r="Q76" t="n">
-        <v>744.9492</v>
+        <v>1</v>
       </c>
       <c r="R76" t="inlineStr">
         <is>
@@ -6857,16 +6857,16 @@
         <v>1</v>
       </c>
       <c r="Q77" t="n">
-        <v>586.803</v>
+        <v>1</v>
       </c>
       <c r="R77" t="inlineStr">
         <is>
-          <t>Tranzact | Watchtower Buyer | APHIX | Carisk Partners | Connatix</t>
+          <t>Tranzact</t>
         </is>
       </c>
       <c r="S77" t="inlineStr">
         <is>
-          <t>Tranzact (Term Loan) | Tranzact (DDTL) | Tranzact (Revolver) | Watchtower Buyer (TL) | Watchtower Buyer (DDTL)</t>
+          <t>Tranzact (Term Loan)</t>
         </is>
       </c>
       <c r="T77" t="b">
@@ -6941,7 +6941,7 @@
         <v>1</v>
       </c>
       <c r="Q78" t="n">
-        <v>694.8678</v>
+        <v>1</v>
       </c>
       <c r="R78" t="inlineStr">
         <is>
@@ -6950,7 +6950,7 @@
       </c>
       <c r="S78" t="inlineStr">
         <is>
-          <t>TransGo (Equity) | TransGo (TL) | TransGo (Revolver)</t>
+          <t>TransGo (Equity)</t>
         </is>
       </c>
       <c r="T78" t="b">
@@ -7004,7 +7004,7 @@
       </c>
       <c r="K79" t="inlineStr">
         <is>
-          <t>STG (TL)</t>
+          <t>STG (Second Out Term Loans)</t>
         </is>
       </c>
       <c r="L79" t="inlineStr">
@@ -7013,28 +7013,28 @@
         </is>
       </c>
       <c r="M79" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="N79" t="b">
         <v>1</v>
       </c>
       <c r="O79" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="P79" t="n">
-        <v>0.76</v>
+        <v>1</v>
       </c>
       <c r="Q79" t="n">
-        <v>883.1317</v>
+        <v>1</v>
       </c>
       <c r="R79" t="inlineStr">
         <is>
-          <t>STG Logistics | Plimpton &amp; Hills | BlackHawk Industrial | WhiteHawk Industrial</t>
+          <t>STG Logistics</t>
         </is>
       </c>
       <c r="S79" t="inlineStr">
         <is>
-          <t>STG (Second Out Term Loans) | STG (First Out New Money Term Loans) | STG (TL) | Plimpton &amp; Hills (TL) | Plimpton &amp; Hills (DDTL)</t>
+          <t>STG (Second Out Term Loans)</t>
         </is>
       </c>
       <c r="T79" t="b">
@@ -7100,10 +7100,10 @@
         <v>0</v>
       </c>
       <c r="N80" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="O80" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="P80" t="n">
         <v>0.9499</v>
@@ -7118,7 +7118,7 @@
       </c>
       <c r="S80" t="inlineStr">
         <is>
-          <t>Sparq (TL) | AKW Holdings (Term Loan) | AKW Holdings (Common) | Sparq (Revolver) | Sparq (Common Equity)</t>
+          <t>Sparq (TL) | Watterson (Revolver) | Dr. Scholl's (Revolver) | AKW Holdings (Term Loan) | AKW Holdings (Common)</t>
         </is>
       </c>
       <c r="T80" t="b">
@@ -7193,16 +7193,16 @@
         <v>1</v>
       </c>
       <c r="Q81" t="n">
-        <v>761.2319</v>
+        <v>1</v>
       </c>
       <c r="R81" t="inlineStr">
         <is>
-          <t>Schlesinger | Global | Insight Global | UniTek | Premiere Global Services (PGi)</t>
+          <t>Schlesinger</t>
         </is>
       </c>
       <c r="S81" t="inlineStr">
         <is>
-          <t>Schlesinger (Equity) | Schlesinger (Term Loan) | UniTek (Common Eq) | Schlesinger (Revolver) | Schlesinger (DDTL)</t>
+          <t>Schlesinger (Equity)</t>
         </is>
       </c>
       <c r="T81" t="b">
@@ -7256,7 +7256,7 @@
       </c>
       <c r="K82" t="inlineStr">
         <is>
-          <t>ProSearch (TL)</t>
+          <t>ProSearch (Revolver)</t>
         </is>
       </c>
       <c r="L82" t="inlineStr">
@@ -7265,28 +7265,28 @@
         </is>
       </c>
       <c r="M82" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="N82" t="b">
         <v>1</v>
       </c>
       <c r="O82" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="P82" t="n">
-        <v>0.9647</v>
+        <v>1</v>
       </c>
       <c r="Q82" t="n">
-        <v>436.6165</v>
+        <v>1</v>
       </c>
       <c r="R82" t="inlineStr">
         <is>
-          <t>ProSearch | Peninsula Pacific Entertainment | None | STG Logistics | Adweek</t>
+          <t>ProSearch</t>
         </is>
       </c>
       <c r="S82" t="inlineStr">
         <is>
-          <t>ProSearch (Revolver) | ProSearch (TL) | ProSearch (DDTL) | Colonial Downs (DDTL) | Datalot (Revolver)</t>
+          <t>ProSearch (Revolver)</t>
         </is>
       </c>
       <c r="T82" t="b">
@@ -7358,19 +7358,19 @@
         <v>1</v>
       </c>
       <c r="P83" t="n">
-        <v>0.901</v>
+        <v>1</v>
       </c>
       <c r="Q83" t="n">
-        <v>454.638</v>
+        <v>1</v>
       </c>
       <c r="R83" t="inlineStr">
         <is>
-          <t>Aechelon | GCOM | QuantiTech | Federal Advisory Partners | Athene</t>
+          <t>Aechelon</t>
         </is>
       </c>
       <c r="S83" t="inlineStr">
         <is>
-          <t>Aechelon (Common Equity) | GCOM (Common Equity) | QuantiTech (Common Equity I) | Federal Advisory Partners (Common Equity) | QuantiTech (Common Equity II)</t>
+          <t>Aechelon (Common Equity)</t>
         </is>
       </c>
       <c r="T83" t="b">
@@ -7445,16 +7445,16 @@
         <v>1</v>
       </c>
       <c r="Q84" t="n">
-        <v>963.2418</v>
+        <v>1</v>
       </c>
       <c r="R84" t="inlineStr">
         <is>
-          <t>BiggerPockets | 48Forty | Harris | Aechelon | Altamira</t>
+          <t>BiggerPockets</t>
         </is>
       </c>
       <c r="S84" t="inlineStr">
         <is>
-          <t>BiggerPockets (Common Equity) | BiggerPockets (TL) | BiggerPockets (Revolver) | 48Forty (Common Equity) | Harris (Common Equity)</t>
+          <t>BiggerPockets (Common Equity)</t>
         </is>
       </c>
       <c r="T84" t="b">
@@ -7494,17 +7494,17 @@
       </c>
       <c r="G85" t="inlineStr">
         <is>
-          <t>Harris</t>
+          <t>C5MI</t>
         </is>
       </c>
       <c r="H85" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I85" t="b">
         <v>1</v>
       </c>
       <c r="J85" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="K85" t="inlineStr">
         <is>
@@ -7526,19 +7526,19 @@
         <v>1</v>
       </c>
       <c r="P85" t="n">
-        <v>0.5929</v>
+        <v>1</v>
       </c>
       <c r="Q85" t="n">
-        <v>389.6323</v>
+        <v>1</v>
       </c>
       <c r="R85" t="inlineStr">
         <is>
-          <t>Harris | BioDerm | C5MI | Cascade | Magnolia</t>
+          <t>C5MI</t>
         </is>
       </c>
       <c r="S85" t="inlineStr">
         <is>
-          <t>C5MI (Preferred Equity) | Harris (Preferred Equity) | BioDerm (Preferred Equity) | Cascade (Preferred Equity) | Magnolia (Preferred Equity)</t>
+          <t>C5MI (Preferred Equity)</t>
         </is>
       </c>
       <c r="T85" t="b">
@@ -7613,16 +7613,16 @@
         <v>1</v>
       </c>
       <c r="Q86" t="n">
-        <v>605.0894</v>
+        <v>1</v>
       </c>
       <c r="R86" t="inlineStr">
         <is>
-          <t>Connatix | Rosco | NORA | RTIC | Rancho Medical</t>
+          <t>Connatix</t>
         </is>
       </c>
       <c r="S86" t="inlineStr">
         <is>
-          <t>Connatix (Common Equity) | Rosco (Common Equity) | NORA (Common Equity) | RTIC (Common Equity) | Rancho (Equity)</t>
+          <t>Connatix (Common Equity)</t>
         </is>
       </c>
       <c r="T86" t="b">
@@ -7697,16 +7697,16 @@
         <v>1</v>
       </c>
       <c r="Q87" t="n">
-        <v>508.5554</v>
+        <v>1</v>
       </c>
       <c r="R87" t="inlineStr">
         <is>
-          <t>Connatix | RTIC | Vertex | Rancho Medical | Rosco</t>
+          <t>Connatix</t>
         </is>
       </c>
       <c r="S87" t="inlineStr">
         <is>
-          <t>Connatix (Common Equity) | Vertex (Preferred Equity) | RTIC (Preferred Equity B) | RTIC (Preferred Equity A) | RTIC (Preferred Equity C)</t>
+          <t>Connatix (Common Equity)</t>
         </is>
       </c>
       <c r="T87" t="b">
@@ -7778,19 +7778,19 @@
         <v>1</v>
       </c>
       <c r="P88" t="n">
-        <v>0.9832</v>
+        <v>1</v>
       </c>
       <c r="Q88" t="n">
-        <v>474.6021</v>
+        <v>1</v>
       </c>
       <c r="R88" t="inlineStr">
         <is>
-          <t>Rancho Medical | Connatix | Rosco | NORA | RTIC</t>
+          <t>Rancho Medical</t>
         </is>
       </c>
       <c r="S88" t="inlineStr">
         <is>
-          <t>Rancho (Equity) | Connatix (Common Equity) | Rosco (Common Equity) | NORA (Common Equity) | RTIC (Common Equity)</t>
+          <t>Rancho (Equity)</t>
         </is>
       </c>
       <c r="T88" t="b">
@@ -7862,19 +7862,19 @@
         <v>1</v>
       </c>
       <c r="P89" t="n">
-        <v>0.992</v>
+        <v>1</v>
       </c>
       <c r="Q89" t="n">
-        <v>657.6972</v>
+        <v>1</v>
       </c>
       <c r="R89" t="inlineStr">
         <is>
-          <t>Tranzact | AKW Holdings | 48Forty | Harris | Aechelon</t>
+          <t>Tranzact</t>
         </is>
       </c>
       <c r="S89" t="inlineStr">
         <is>
-          <t>Tranzact (Common Equity) | Tranzact (DDTL) | Tranzact (Revolver) | Tranzact (Term Loan) | AKW Holdings (Common)</t>
+          <t>Tranzact (Common Equity)</t>
         </is>
       </c>
       <c r="T89" t="b">
@@ -7946,19 +7946,19 @@
         <v>1</v>
       </c>
       <c r="P90" t="n">
-        <v>0.8658</v>
+        <v>1</v>
       </c>
       <c r="Q90" t="n">
-        <v>357.3443</v>
+        <v>1</v>
       </c>
       <c r="R90" t="inlineStr">
         <is>
-          <t>Tyto Athene | AKW Holdings | 48Forty | Harris | Aechelon</t>
+          <t>Tyto Athene</t>
         </is>
       </c>
       <c r="S90" t="inlineStr">
         <is>
-          <t>Tyto Athene (Equity) | AKW Holdings (Common) | Tyto Athene (Pref) | 48Forty (Common Equity) | Harris (Common Equity)</t>
+          <t>Tyto Athene (Equity)</t>
         </is>
       </c>
       <c r="T90" t="b">
@@ -8030,19 +8030,19 @@
         <v>1</v>
       </c>
       <c r="P91" t="n">
-        <v>0.8658</v>
+        <v>1</v>
       </c>
       <c r="Q91" t="n">
-        <v>341.3221</v>
+        <v>1</v>
       </c>
       <c r="R91" t="inlineStr">
         <is>
-          <t>Tyto Athene | AKW Holdings | Harris | BioDerm | C5MI</t>
+          <t>Tyto Athene</t>
         </is>
       </c>
       <c r="S91" t="inlineStr">
         <is>
-          <t>Tyto Athene (Pref) | BioDerm (Preferred Equity) | Harris (Preferred Equity) | Tyto Athene (Equity) | C5MI (Preferred Equity)</t>
+          <t>Tyto Athene (Pref)</t>
         </is>
       </c>
       <c r="T91" t="b">
@@ -8114,19 +8114,19 @@
         <v>1</v>
       </c>
       <c r="P92" t="n">
-        <v>0.928</v>
+        <v>1</v>
       </c>
       <c r="Q92" t="n">
-        <v>495.753</v>
+        <v>1</v>
       </c>
       <c r="R92" t="inlineStr">
         <is>
-          <t>Vertex | Connatix | Rosco | NORA | RTIC</t>
+          <t>Vertex</t>
         </is>
       </c>
       <c r="S92" t="inlineStr">
         <is>
-          <t>Vertex (Common Equity) | Vertex (Preferred Equity) | NORA (Common Equity) | RTIC (Common Equity) | Connatix (Common Equity)</t>
+          <t>Vertex (Common Equity)</t>
         </is>
       </c>
       <c r="T92" t="b">
@@ -8198,19 +8198,19 @@
         <v>1</v>
       </c>
       <c r="P93" t="n">
-        <v>0.9332</v>
+        <v>1</v>
       </c>
       <c r="Q93" t="n">
-        <v>566.9647</v>
+        <v>1</v>
       </c>
       <c r="R93" t="inlineStr">
         <is>
-          <t>Vertex | RTIC | Rancho Medical | Connatix | Rosco</t>
+          <t>Vertex</t>
         </is>
       </c>
       <c r="S93" t="inlineStr">
         <is>
-          <t>Vertex (Preferred Equity) | RTIC (Preferred Equity B) | RTIC (Preferred Equity A) | Vertex (Common Equity) | RTIC (Preferred Equity C)</t>
+          <t>Vertex (Preferred Equity)</t>
         </is>
       </c>
       <c r="T93" t="b">
@@ -8245,23 +8245,21 @@
       </c>
       <c r="F94" t="inlineStr">
         <is>
+          <t>Watchtower</t>
+        </is>
+      </c>
+      <c r="G94" t="inlineStr">
+        <is>
           <t>Watchtower Holdings</t>
-        </is>
-      </c>
-      <c r="G94" t="inlineStr">
-        <is>
-          <t>Watchtower</t>
         </is>
       </c>
       <c r="H94" t="b">
         <v>0</v>
       </c>
       <c r="I94" t="b">
-        <v>1</v>
-      </c>
-      <c r="J94" t="n">
-        <v>2</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="J94" t="inlineStr"/>
       <c r="K94" t="inlineStr">
         <is>
           <t>Watchtower Holding (Common Equity)</t>
@@ -8285,16 +8283,16 @@
         <v>1</v>
       </c>
       <c r="Q94" t="n">
-        <v>495.1412</v>
+        <v>1</v>
       </c>
       <c r="R94" t="inlineStr">
         <is>
-          <t>Watchtower | Watchtower Holdings | Watchtower Buyer | AKW Holdings | 48Forty</t>
+          <t>Watchtower Holdings</t>
         </is>
       </c>
       <c r="S94" t="inlineStr">
         <is>
-          <t>Watchtower Holding (Common Equity) | AKW Holdings (Common) | 48Forty (Common Equity) | Watchtower (TL) | Watchtower (Revolver)</t>
+          <t>Watchtower Holding (Common Equity)</t>
         </is>
       </c>
       <c r="T94" t="b">
@@ -8369,16 +8367,16 @@
         <v>1</v>
       </c>
       <c r="Q95" t="n">
-        <v>690.3403</v>
+        <v>1</v>
       </c>
       <c r="R95" t="inlineStr">
         <is>
-          <t>Watterson | AKW Holdings | 48Forty | Harris | Aechelon</t>
+          <t>Watterson</t>
         </is>
       </c>
       <c r="S95" t="inlineStr">
         <is>
-          <t>Watterson (Equity) | Watterson (TL) | Watterson (Revolver) | Watterson (DDTL) | AKW Holdings (Common)</t>
+          <t>Watterson (Equity)</t>
         </is>
       </c>
       <c r="T95" t="b">
@@ -8503,25 +8501,25 @@
         </is>
       </c>
       <c r="I2" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="J2" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t>66.7%</t>
+          <t>88.9%</t>
         </is>
       </c>
       <c r="L2" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="M2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="N2" t="inlineStr">
         <is>
-          <t>100.0%</t>
+          <t>88.9%</t>
         </is>
       </c>
     </row>
@@ -8535,25 +8533,25 @@
         <v>13</v>
       </c>
       <c r="C3" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="D3" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>84.6%</t>
+          <t>92.3%</t>
         </is>
       </c>
       <c r="F3" t="n">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="G3" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>100.0%</t>
+          <t>92.3%</t>
         </is>
       </c>
       <c r="I3" t="n">
@@ -8751,14 +8749,14 @@
         <v>18</v>
       </c>
       <c r="C7" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="D7" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>72.2%</t>
+          <t>77.8%</t>
         </is>
       </c>
       <c r="F7" t="n">
@@ -8773,14 +8771,14 @@
         </is>
       </c>
       <c r="I7" t="n">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="J7" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="K7" t="inlineStr">
         <is>
-          <t>55.6%</t>
+          <t>66.7%</t>
         </is>
       </c>
       <c r="L7" t="n">

</xml_diff>

<commit_message>
batch test concurrent test
</commit_message>
<xml_diff>
--- a/evaluation_results.xlsx
+++ b/evaluation_results.xlsx
@@ -1599,12 +1599,12 @@
       </c>
       <c r="R14" t="inlineStr">
         <is>
-          <t>Centauri Health | Watchtower Buyer | 360DG | Integrated Data Services | Tranzact</t>
+          <t>Centauri Health | Watchtower Buyer | APHIX | Carisk Partners | Connatix</t>
         </is>
       </c>
       <c r="S14" t="inlineStr">
         <is>
-          <t>Centauri Health (TL) | Centauri Health (Revolver) | Watchtower Buyer (Revolver) | Centauri Health (DDTL) | 360DG (Revolver)</t>
+          <t>Centauri Health (TL) | Centauri Health (Revolver) | Watchtower Buyer (Revolver) | Centauri Health (DDTL) | Carisk Partners (Revolver)</t>
         </is>
       </c>
       <c r="T14" t="b">

</xml_diff>

<commit_message>
Knowledge match case test
</commit_message>
<xml_diff>
--- a/evaluation_results.xlsx
+++ b/evaluation_results.xlsx
@@ -1589,10 +1589,10 @@
         <v>1</v>
       </c>
       <c r="O14" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="P14" t="n">
-        <v>0.9533</v>
+        <v>1</v>
       </c>
       <c r="Q14" t="n">
         <v>345.8854</v>
@@ -1604,7 +1604,7 @@
       </c>
       <c r="S14" t="inlineStr">
         <is>
-          <t>Centauri Health (TL) | Centauri Health (Revolver) | Watchtower Buyer (Revolver) | Centauri Health (DDTL) | Carisk Partners (Revolver)</t>
+          <t>Centauri Health (TL) | Watchtower Buyer (Revolver) | Centauri Health (Revolver) | Centauri Health (DDTL) | Centauri Health (Equity)</t>
         </is>
       </c>
       <c r="T14" t="b">
@@ -2264,10 +2264,10 @@
         <v>5</v>
       </c>
       <c r="P22" t="n">
-        <v>0.8537</v>
+        <v>0.8538</v>
       </c>
       <c r="Q22" t="n">
-        <v>86.6747</v>
+        <v>87.51949999999999</v>
       </c>
       <c r="R22" t="inlineStr">
         <is>
@@ -2730,16 +2730,18 @@
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>AKW Holdings</t>
+          <t>Fairbanks Morse Defense</t>
         </is>
       </c>
       <c r="H28" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I28" t="b">
-        <v>0</v>
-      </c>
-      <c r="J28" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="J28" t="n">
+        <v>1</v>
+      </c>
       <c r="K28" t="inlineStr">
         <is>
           <t>Fairbanks Morse Defense (Term Loan)</t>
@@ -2747,30 +2749,32 @@
       </c>
       <c r="L28" t="inlineStr">
         <is>
-          <t>AKW Holdings (Term Loan)</t>
+          <t>Fairbanks Morse Defense (Term Loan)</t>
         </is>
       </c>
       <c r="M28" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="N28" t="b">
-        <v>0</v>
-      </c>
-      <c r="O28" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="O28" t="n">
+        <v>1</v>
+      </c>
       <c r="P28" t="n">
-        <v>0.5628</v>
+        <v>1</v>
       </c>
       <c r="Q28" t="n">
-        <v>36.6381</v>
+        <v>1</v>
       </c>
       <c r="R28" t="inlineStr">
         <is>
-          <t>AKW Holdings</t>
+          <t>Fairbanks Morse Defense</t>
         </is>
       </c>
       <c r="S28" t="inlineStr">
         <is>
-          <t>AKW Holdings (Term Loan) | AKW Holdings (Common)</t>
+          <t>Fairbanks Morse Defense (Term Loan)</t>
         </is>
       </c>
       <c r="T28" t="b">
@@ -2925,7 +2929,7 @@
         <v>1</v>
       </c>
       <c r="Q30" t="n">
-        <v>435.0036</v>
+        <v>434.7123</v>
       </c>
       <c r="R30" t="inlineStr">
         <is>
@@ -3058,17 +3062,17 @@
       </c>
       <c r="G32" t="inlineStr">
         <is>
-          <t>APT Healthcare</t>
+          <t>The Creative Group</t>
         </is>
       </c>
       <c r="H32" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I32" t="b">
         <v>1</v>
       </c>
       <c r="J32" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="K32" t="inlineStr">
         <is>
@@ -3077,32 +3081,32 @@
       </c>
       <c r="L32" t="inlineStr">
         <is>
-          <t>APT Healthcare (Incr. DDTL)</t>
+          <t>The Creative Group (Term Loan)</t>
         </is>
       </c>
       <c r="M32" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="N32" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O32" t="n">
-        <v>15</v>
+        <v>1</v>
       </c>
       <c r="P32" t="n">
-        <v>0.7469</v>
+        <v>1</v>
       </c>
       <c r="Q32" t="n">
-        <v>396.0039</v>
+        <v>1</v>
       </c>
       <c r="R32" t="inlineStr">
         <is>
-          <t>APT Healthcare | Lilly Lashes | Zips | The Creative Group | The Original Cakerie</t>
+          <t>The Creative Group</t>
         </is>
       </c>
       <c r="S32" t="inlineStr">
         <is>
-          <t>APT Healthcare (Incr. DDTL) | Zips (DDTL) | Bland Landscaping (DDTL) | AFC Industries (DDTL) | Carnegie Dartlet (DDTL)</t>
+          <t>The Creative Group (Term Loan)</t>
         </is>
       </c>
       <c r="T32" t="b">
@@ -3142,16 +3146,18 @@
       </c>
       <c r="G33" t="inlineStr">
         <is>
-          <t>Boss Industries</t>
+          <t>360DG</t>
         </is>
       </c>
       <c r="H33" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I33" t="b">
-        <v>0</v>
-      </c>
-      <c r="J33" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="J33" t="n">
+        <v>1</v>
+      </c>
       <c r="K33" t="inlineStr">
         <is>
           <t>360DG (DDTL A)</t>
@@ -3159,30 +3165,32 @@
       </c>
       <c r="L33" t="inlineStr">
         <is>
-          <t>AFC Industries (DDTL)</t>
+          <t>360DG (DDTL A)</t>
         </is>
       </c>
       <c r="M33" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="N33" t="b">
-        <v>0</v>
-      </c>
-      <c r="O33" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="O33" t="n">
+        <v>1</v>
+      </c>
       <c r="P33" t="n">
-        <v>0.8363</v>
+        <v>1</v>
       </c>
       <c r="Q33" t="n">
-        <v>399.9936</v>
+        <v>1</v>
       </c>
       <c r="R33" t="inlineStr">
         <is>
-          <t>Boss Industries | ECM Industries | AFC Acquisitions | DermaRite | Nsi Industries</t>
+          <t>360DG</t>
         </is>
       </c>
       <c r="S33" t="inlineStr">
         <is>
-          <t>AFC Industries (DDTL) | Nsi Industries (DDTL) | AFC Industries (TL) | Boss Industries (Term Loan) | ECM Industries (TL)</t>
+          <t>360DG (DDTL A)</t>
         </is>
       </c>
       <c r="T33" t="b">
@@ -3978,16 +3986,18 @@
       </c>
       <c r="G43" t="inlineStr">
         <is>
-          <t>TVC</t>
+          <t>A1 Garage</t>
         </is>
       </c>
       <c r="H43" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I43" t="b">
-        <v>0</v>
-      </c>
-      <c r="J43" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="J43" t="n">
+        <v>1</v>
+      </c>
       <c r="K43" t="inlineStr">
         <is>
           <t>A1 Garage (DDTL)</t>
@@ -3995,30 +4005,32 @@
       </c>
       <c r="L43" t="inlineStr">
         <is>
-          <t>US Fertility (DDTL)</t>
+          <t>A1 Garage (DDTL)</t>
         </is>
       </c>
       <c r="M43" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="N43" t="b">
-        <v>0</v>
-      </c>
-      <c r="O43" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="O43" t="n">
+        <v>1</v>
+      </c>
       <c r="P43" t="n">
-        <v>0.7544</v>
+        <v>1</v>
       </c>
       <c r="Q43" t="n">
-        <v>396.3347</v>
+        <v>1</v>
       </c>
       <c r="R43" t="inlineStr">
         <is>
-          <t>TVC | US Fertility</t>
+          <t>A1 Garage</t>
         </is>
       </c>
       <c r="S43" t="inlineStr">
         <is>
-          <t>US Fertility (DDTL) | TVC (DDTL) | TVC (TL) | US Fertility (Term Loan) | Bland Landscaping (DDTL)</t>
+          <t>A1 Garage (DDTL)</t>
         </is>
       </c>
       <c r="T43" t="b">
@@ -4058,16 +4070,18 @@
       </c>
       <c r="G44" t="inlineStr">
         <is>
-          <t>TVC</t>
+          <t>A1 Garage</t>
         </is>
       </c>
       <c r="H44" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I44" t="b">
-        <v>0</v>
-      </c>
-      <c r="J44" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="J44" t="n">
+        <v>1</v>
+      </c>
       <c r="K44" t="inlineStr">
         <is>
           <t>A1 Garage (Term Loan)</t>
@@ -4075,30 +4089,32 @@
       </c>
       <c r="L44" t="inlineStr">
         <is>
-          <t>TVC (TL)</t>
+          <t>A1 Garage (Term Loan)</t>
         </is>
       </c>
       <c r="M44" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="N44" t="b">
-        <v>0</v>
-      </c>
-      <c r="O44" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="O44" t="n">
+        <v>1</v>
+      </c>
       <c r="P44" t="n">
-        <v>0.7544</v>
+        <v>1</v>
       </c>
       <c r="Q44" t="n">
-        <v>294.2774</v>
+        <v>1</v>
       </c>
       <c r="R44" t="inlineStr">
         <is>
-          <t>TVC | US Fertility</t>
+          <t>A1 Garage</t>
         </is>
       </c>
       <c r="S44" t="inlineStr">
         <is>
-          <t>TVC (TL) | US Fertility (Term Loan) | US Fertility (DDTL) | TVC (DDTL) | MeritDirect (Term Loan)</t>
+          <t>A1 Garage (Term Loan)</t>
         </is>
       </c>
       <c r="T44" t="b">
@@ -4164,16 +4180,16 @@
         <v>0</v>
       </c>
       <c r="N45" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="O45" t="n">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="P45" t="n">
         <v>0.999</v>
       </c>
       <c r="Q45" t="n">
-        <v>591.8692</v>
+        <v>591.5267</v>
       </c>
       <c r="R45" t="inlineStr">
         <is>
@@ -4182,7 +4198,7 @@
       </c>
       <c r="S45" t="inlineStr">
         <is>
-          <t>Aeronix (DDTL) | Aeronix (Common Equity) | AKW Holdings (Term Loan) | Aeronix (TL) | 4Wall Entertainment (Term Loan)</t>
+          <t>Aeronix (DDTL) | Aeronix (Common Equity) | AKW Holdings (Term Loan) | 4Wall Entertainment (Term Loan) | Dr. Scholl's (Term Loan)</t>
         </is>
       </c>
       <c r="T45" t="b">
@@ -4390,16 +4406,18 @@
       </c>
       <c r="G48" t="inlineStr">
         <is>
-          <t>Simplicity Group</t>
+          <t>Smartronix / Trident</t>
         </is>
       </c>
       <c r="H48" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I48" t="b">
-        <v>0</v>
-      </c>
-      <c r="J48" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="J48" t="n">
+        <v>1</v>
+      </c>
       <c r="K48" t="inlineStr">
         <is>
           <t>Smartronix / Trident (TL)</t>
@@ -4407,30 +4425,32 @@
       </c>
       <c r="L48" t="inlineStr">
         <is>
-          <t>STV Group (TL)</t>
+          <t>Smartronix / Trident (TL)</t>
         </is>
       </c>
       <c r="M48" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="N48" t="b">
-        <v>0</v>
-      </c>
-      <c r="O48" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="O48" t="n">
+        <v>1</v>
+      </c>
       <c r="P48" t="n">
-        <v>0.5505</v>
+        <v>1</v>
       </c>
       <c r="Q48" t="n">
-        <v>235.981</v>
+        <v>1</v>
       </c>
       <c r="R48" t="inlineStr">
         <is>
-          <t>Simplicity Group | None | Case Works Group | Guild Garage Group | STV Group</t>
+          <t>Smartronix / Trident</t>
         </is>
       </c>
       <c r="S48" t="inlineStr">
         <is>
-          <t>STV Group (TL) | Simplicity Group (TL) | Case Works Group (Term Loan) | Guild Garage Group (Term Loan) | Simplicity Group (DDTL)</t>
+          <t>Smartronix / Trident (TL)</t>
         </is>
       </c>
       <c r="T48" t="b">
@@ -4589,7 +4609,7 @@
         <v>1</v>
       </c>
       <c r="Q50" t="n">
-        <v>672.4636</v>
+        <v>672.6747</v>
       </c>
       <c r="R50" t="inlineStr">
         <is>
@@ -5849,7 +5869,7 @@
         <v>1</v>
       </c>
       <c r="Q65" t="n">
-        <v>873.5107</v>
+        <v>875.8619</v>
       </c>
       <c r="R65" t="inlineStr">
         <is>
@@ -5858,7 +5878,7 @@
       </c>
       <c r="S65" t="inlineStr">
         <is>
-          <t>4Wall Entertainment (Revolver) | 4Wall Entertainment (Term Loan) | 4Wall Entertainment (DDTL) | ECL Entertainment (Term Loan) | Peninsula Pacific Entertainment (Term Loan B)</t>
+          <t>4Wall Entertainment (Revolver) | 4Wall Entertainment (Term Loan) | 4Wall Entertainment (DDTL)</t>
         </is>
       </c>
       <c r="T65" t="b">
@@ -5933,7 +5953,7 @@
         <v>1</v>
       </c>
       <c r="Q66" t="n">
-        <v>546.4172</v>
+        <v>547.049</v>
       </c>
       <c r="R66" t="inlineStr">
         <is>
@@ -6017,7 +6037,7 @@
         <v>1</v>
       </c>
       <c r="Q67" t="n">
-        <v>1005.7311</v>
+        <v>1008.9297</v>
       </c>
       <c r="R67" t="inlineStr">
         <is>
@@ -6101,7 +6121,7 @@
         <v>1</v>
       </c>
       <c r="Q68" t="n">
-        <v>1005.7311</v>
+        <v>1008.9297</v>
       </c>
       <c r="R68" t="inlineStr">
         <is>
@@ -6185,7 +6205,7 @@
         <v>1</v>
       </c>
       <c r="Q69" t="n">
-        <v>746.6063</v>
+        <v>748.769</v>
       </c>
       <c r="R69" t="inlineStr">
         <is>
@@ -6194,7 +6214,7 @@
       </c>
       <c r="S69" t="inlineStr">
         <is>
-          <t>Cano Health (Equity) | Cano Health (Term Loan) | Ro Health (Revolver) | Confluent Health (TL) | Ro Health (Term Loan)</t>
+          <t>Cano Health (Equity) | Centauri Health (TL) | Comprehensive Rehab Consultants (Revolver)</t>
         </is>
       </c>
       <c r="T69" t="b">
@@ -6353,7 +6373,7 @@
         <v>1</v>
       </c>
       <c r="Q71" t="n">
-        <v>949.814</v>
+        <v>952.9135</v>
       </c>
       <c r="R71" t="inlineStr">
         <is>
@@ -6434,10 +6454,10 @@
         <v>3</v>
       </c>
       <c r="P72" t="n">
-        <v>0.9471000000000001</v>
+        <v>0.9472</v>
       </c>
       <c r="Q72" t="n">
-        <v>524.371</v>
+        <v>525.5556</v>
       </c>
       <c r="R72" t="inlineStr">
         <is>
@@ -7100,13 +7120,13 @@
         <v>0</v>
       </c>
       <c r="N80" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O80" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="P80" t="n">
-        <v>0.9499</v>
+        <v>1</v>
       </c>
       <c r="Q80" t="n">
         <v>382.3594</v>
@@ -7118,7 +7138,7 @@
       </c>
       <c r="S80" t="inlineStr">
         <is>
-          <t>Sparq (TL) | Watterson (Revolver) | Dr. Scholl's (Revolver) | AKW Holdings (Term Loan) | AKW Holdings (Common)</t>
+          <t>Sparq (TL) | Watterson (Revolver) | Dr. Scholl's (Revolver) | Sparq (Revolver) | Sparq (Common Equity)</t>
         </is>
       </c>
       <c r="T80" t="b">
@@ -8512,14 +8532,14 @@
         </is>
       </c>
       <c r="L2" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="M2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="N2" t="inlineStr">
         <is>
-          <t>88.9%</t>
+          <t>100.0%</t>
         </is>
       </c>
     </row>
@@ -8695,47 +8715,47 @@
         <v>31</v>
       </c>
       <c r="C6" t="n">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="D6" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>90.3%</t>
+          <t>96.8%</t>
         </is>
       </c>
       <c r="F6" t="n">
+        <v>30</v>
+      </c>
+      <c r="G6" t="n">
+        <v>1</v>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>96.8%</t>
+        </is>
+      </c>
+      <c r="I6" t="n">
+        <v>27</v>
+      </c>
+      <c r="J6" t="n">
+        <v>4</v>
+      </c>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>87.1%</t>
+        </is>
+      </c>
+      <c r="L6" t="n">
         <v>29</v>
       </c>
-      <c r="G6" t="n">
+      <c r="M6" t="n">
         <v>2</v>
       </c>
-      <c r="H6" t="inlineStr">
+      <c r="N6" t="inlineStr">
         <is>
           <t>93.5%</t>
-        </is>
-      </c>
-      <c r="I6" t="n">
-        <v>25</v>
-      </c>
-      <c r="J6" t="n">
-        <v>6</v>
-      </c>
-      <c r="K6" t="inlineStr">
-        <is>
-          <t>80.6%</t>
-        </is>
-      </c>
-      <c r="L6" t="n">
-        <v>27</v>
-      </c>
-      <c r="M6" t="n">
-        <v>4</v>
-      </c>
-      <c r="N6" t="inlineStr">
-        <is>
-          <t>87.1%</t>
         </is>
       </c>
     </row>
@@ -8749,47 +8769,47 @@
         <v>18</v>
       </c>
       <c r="C7" t="n">
-        <v>14</v>
+        <v>18</v>
       </c>
       <c r="D7" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>77.8%</t>
+          <t>100.0%</t>
         </is>
       </c>
       <c r="F7" t="n">
-        <v>14</v>
+        <v>18</v>
       </c>
       <c r="G7" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>77.8%</t>
+          <t>100.0%</t>
         </is>
       </c>
       <c r="I7" t="n">
-        <v>12</v>
+        <v>16</v>
       </c>
       <c r="J7" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="K7" t="inlineStr">
         <is>
-          <t>66.7%</t>
+          <t>88.9%</t>
         </is>
       </c>
       <c r="L7" t="n">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="M7" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="N7" t="inlineStr">
         <is>
-          <t>77.8%</t>
+          <t>94.4%</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
fixed array input and config usage in function app removed unnecessary mapped fields search
</commit_message>
<xml_diff>
--- a/evaluation_results.xlsx
+++ b/evaluation_results.xlsx
@@ -1500,11 +1500,7 @@
           <t>Lightspeed Buyer VT1 R/C</t>
         </is>
       </c>
-      <c r="E14" t="inlineStr">
-        <is>
-          <t>lightspeed buyer</t>
-        </is>
-      </c>
+      <c r="E14" t="inlineStr"/>
       <c r="F14" t="inlineStr">
         <is>
           <t>Centauri Health</t>
@@ -2144,11 +2140,7 @@
           <t>OSG Topco Holdings LLC - Class A Unit</t>
         </is>
       </c>
-      <c r="E22" t="inlineStr">
-        <is>
-          <t>osg topco holdings class a unit</t>
-        </is>
-      </c>
+      <c r="E22" t="inlineStr"/>
       <c r="F22" t="inlineStr">
         <is>
           <t>OSG Billing Services</t>
@@ -2156,11 +2148,11 @@
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>OSG Billing Services</t>
+          <t>U.S. Well</t>
         </is>
       </c>
       <c r="H22" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I22" t="b">
         <v>1</v>
@@ -2188,7 +2180,7 @@
         <v>5</v>
       </c>
       <c r="P22" t="n">
-        <v>0.8538</v>
+        <v>0.6781</v>
       </c>
       <c r="Q22" t="n">
         <v>0.7006573962868813</v>
@@ -2788,11 +2780,7 @@
           <t>PlayPower T/L (5/19)</t>
         </is>
       </c>
-      <c r="E30" t="inlineStr">
-        <is>
-          <t>playpower</t>
-        </is>
-      </c>
+      <c r="E30" t="inlineStr"/>
       <c r="F30" t="inlineStr">
         <is>
           <t>Planview</t>
@@ -3988,11 +3976,7 @@
           <t>SV-Aero Holdings LLC Term Loan</t>
         </is>
       </c>
-      <c r="E45" t="inlineStr">
-        <is>
-          <t>sv aero holdings</t>
-        </is>
-      </c>
+      <c r="E45" t="inlineStr"/>
       <c r="F45" t="inlineStr">
         <is>
           <t>Aeronix</t>
@@ -4392,11 +4376,7 @@
           <t>Zips Car Wash LLC Roll Up Term Loan</t>
         </is>
       </c>
-      <c r="E50" t="inlineStr">
-        <is>
-          <t>zips car wash</t>
-        </is>
-      </c>
+      <c r="E50" t="inlineStr"/>
       <c r="F50" t="inlineStr">
         <is>
           <t>Zips</t>
@@ -5516,11 +5496,7 @@
           <t>MidOcean JF Holdings Corp. 5th Amendment Term Loan</t>
         </is>
       </c>
-      <c r="E64" t="inlineStr">
-        <is>
-          <t>midocean jf holdings</t>
-        </is>
-      </c>
+      <c r="E64" t="inlineStr"/>
       <c r="F64" t="inlineStr">
         <is>
           <t>Jones &amp; Frank</t>
@@ -5600,11 +5576,7 @@
           <t>4Wall Entertainment</t>
         </is>
       </c>
-      <c r="E65" t="inlineStr">
-        <is>
-          <t>4wall entertainment</t>
-        </is>
-      </c>
+      <c r="E65" t="inlineStr"/>
       <c r="F65" t="inlineStr">
         <is>
           <t>4Wall Entertainment</t>
@@ -5684,11 +5656,7 @@
           <t>Aeronix</t>
         </is>
       </c>
-      <c r="E66" t="inlineStr">
-        <is>
-          <t>aeronix</t>
-        </is>
-      </c>
+      <c r="E66" t="inlineStr"/>
       <c r="F66" t="inlineStr">
         <is>
           <t>Aeronix</t>
@@ -5768,11 +5736,7 @@
           <t>Any Hour Services</t>
         </is>
       </c>
-      <c r="E67" t="inlineStr">
-        <is>
-          <t>any hour services</t>
-        </is>
-      </c>
+      <c r="E67" t="inlineStr"/>
       <c r="F67" t="inlineStr">
         <is>
           <t>Any Hour Services</t>
@@ -5852,11 +5816,7 @@
           <t>Any Hour Services</t>
         </is>
       </c>
-      <c r="E68" t="inlineStr">
-        <is>
-          <t>any hour services</t>
-        </is>
-      </c>
+      <c r="E68" t="inlineStr"/>
       <c r="F68" t="inlineStr">
         <is>
           <t>Any Hour Services</t>
@@ -5936,11 +5896,7 @@
           <t>Cano Health</t>
         </is>
       </c>
-      <c r="E69" t="inlineStr">
-        <is>
-          <t>cano health</t>
-        </is>
-      </c>
+      <c r="E69" t="inlineStr"/>
       <c r="F69" t="inlineStr">
         <is>
           <t>Cano Health</t>
@@ -6100,11 +6056,7 @@
           <t>Infinity Home Services</t>
         </is>
       </c>
-      <c r="E71" t="inlineStr">
-        <is>
-          <t>infinity home services</t>
-        </is>
-      </c>
+      <c r="E71" t="inlineStr"/>
       <c r="F71" t="inlineStr">
         <is>
           <t>Infinity Home Services</t>
@@ -6184,11 +6136,7 @@
           <t>KNS</t>
         </is>
       </c>
-      <c r="E72" t="inlineStr">
-        <is>
-          <t>kns</t>
-        </is>
-      </c>
+      <c r="E72" t="inlineStr"/>
       <c r="F72" t="inlineStr">
         <is>
           <t>KNS</t>
@@ -6828,11 +6776,7 @@
           <t>Rural Sourcing Holdings, Inc. - Unfunded Revolver</t>
         </is>
       </c>
-      <c r="E80" t="inlineStr">
-        <is>
-          <t>rural sourcing holdings</t>
-        </is>
-      </c>
+      <c r="E80" t="inlineStr"/>
       <c r="F80" t="inlineStr">
         <is>
           <t>Sparq</t>
@@ -8403,14 +8347,14 @@
         <v>31</v>
       </c>
       <c r="C6" t="n">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="D6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>96.8%</t>
+          <t>93.5%</t>
         </is>
       </c>
       <c r="F6" t="n">

</xml_diff>